<commit_message>
MAJ pipeline 2026-07-29 08:04
</commit_message>
<xml_diff>
--- a/jira_export_2026-07-29.xlsx
+++ b/jira_export_2026-07-29.xlsx
@@ -723,7 +723,7 @@
     <row r="7" ht="26" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>60,145 €</t>
+          <t>60,599 €</t>
         </is>
       </c>
       <c r="B7" s="7" t="n"/>
@@ -737,7 +737,7 @@
       <c r="F7" s="7" t="n"/>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>63.3%</t>
+          <t>63.8%</t>
         </is>
       </c>
       <c r="H7" s="7" t="n"/>
@@ -763,14 +763,14 @@
     <row r="11" ht="26" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>22,046 €</t>
+          <t>22,306 €</t>
         </is>
       </c>
       <c r="B11" s="7" t="n"/>
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>38,098 €</t>
+          <t>38,293 €</t>
         </is>
       </c>
       <c r="E11" s="7" t="n"/>
@@ -818,7 +818,7 @@
     <row r="16" ht="26" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>547 h</t>
+          <t>558 h</t>
         </is>
       </c>
       <c r="B16" s="7" t="n"/>
@@ -832,7 +832,7 @@
       <c r="F16" s="7" t="n"/>
       <c r="G16" s="8" t="inlineStr">
         <is>
-          <t>68.5%</t>
+          <t>69.9%</t>
         </is>
       </c>
       <c r="H16" s="7" t="n"/>
@@ -936,7 +936,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P186"/>
+  <dimension ref="A1:P187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="43" customWidth="1" min="1" max="1"/>
@@ -3160,7 +3160,7 @@
         <v>1</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L34" s="14" t="inlineStr">
         <is>
@@ -3179,7 +3179,7 @@
         <v>870.03</v>
       </c>
       <c r="P34" s="15" t="n">
-        <v>87</v>
+        <v>79.09</v>
       </c>
     </row>
     <row r="35">
@@ -3749,13 +3749,13 @@
         </is>
       </c>
       <c r="N42" s="15" t="n">
-        <v>1365</v>
+        <v>0</v>
       </c>
       <c r="O42" s="15" t="n">
-        <v>1560</v>
+        <v>1755</v>
       </c>
       <c r="P42" s="15" t="n">
-        <v>567.27</v>
+        <v>638.1799999999999</v>
       </c>
     </row>
     <row r="43">
@@ -6104,7 +6104,7 @@
         <v>3</v>
       </c>
       <c r="K75" s="11" t="n">
-        <v>1.75</v>
+        <v>3.25</v>
       </c>
       <c r="L75" s="11" t="inlineStr">
         <is>
@@ -6120,10 +6120,10 @@
         <v>548.4</v>
       </c>
       <c r="O75" s="16" t="n">
-        <v>0</v>
+        <v>109.68</v>
       </c>
       <c r="P75" s="12" t="n">
-        <v>0</v>
+        <v>33.75</v>
       </c>
     </row>
     <row r="76">
@@ -6405,7 +6405,7 @@
         </is>
       </c>
       <c r="N79" s="12" t="n">
-        <v>882.5</v>
+        <v>0</v>
       </c>
       <c r="O79" s="12" t="n">
         <v>882.5</v>
@@ -9614,7 +9614,7 @@
         <v>8</v>
       </c>
       <c r="K124" s="14" t="n">
-        <v>4.5</v>
+        <v>6</v>
       </c>
       <c r="L124" s="14" t="inlineStr">
         <is>
@@ -11624,7 +11624,7 @@
         <v>16</v>
       </c>
       <c r="K153" s="11" t="n">
-        <v>2.25</v>
+        <v>2.5</v>
       </c>
       <c r="L153" s="11" t="inlineStr"/>
       <c r="M153" s="11" t="inlineStr"/>
@@ -12812,7 +12812,7 @@
         <v>30</v>
       </c>
       <c r="K171" s="11" t="n">
-        <v>7.75</v>
+        <v>8</v>
       </c>
       <c r="L171" s="11" t="inlineStr"/>
       <c r="M171" s="11" t="inlineStr"/>
@@ -12936,7 +12936,7 @@
         <v>34</v>
       </c>
       <c r="K173" s="11" t="n">
-        <v>10.5</v>
+        <v>11.5</v>
       </c>
       <c r="L173" s="11" t="inlineStr">
         <is>
@@ -13071,7 +13071,11 @@
           <t>PDMDEP-34532</t>
         </is>
       </c>
-      <c r="M175" s="11" t="inlineStr"/>
+      <c r="M175" s="11" t="inlineStr">
+        <is>
+          <t>412263</t>
+        </is>
+      </c>
       <c r="N175" s="12" t="n">
         <v>0</v>
       </c>
@@ -13335,18 +13339,18 @@
     <row r="180">
       <c r="A180" s="13" t="inlineStr">
         <is>
-          <t>PSC-1270</t>
+          <t>PSC-1283</t>
         </is>
       </c>
       <c r="B180" s="14" t="inlineStr">
         <is>
-          <t>COMMUNE DE CASTELNAUDARY</t>
+          <t>MAIRIE DE ANNET SUR MARNE</t>
         </is>
       </c>
       <c r="C180" s="14" t="inlineStr"/>
       <c r="D180" s="14" t="inlineStr">
         <is>
-          <t>COMMUNE DE CASTELNAUDARY</t>
+          <t>MAIRIE DE ANNET SUR MARNE</t>
         </is>
       </c>
       <c r="E180" s="14" t="inlineStr"/>
@@ -13363,7 +13367,7 @@
       <c r="H180" s="14" t="inlineStr"/>
       <c r="I180" s="14" t="inlineStr">
         <is>
-          <t>19/05/2026</t>
+          <t>28/05/2026</t>
         </is>
       </c>
       <c r="J180" s="14" t="n">
@@ -13374,19 +13378,19 @@
       </c>
       <c r="L180" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-33362</t>
+          <t>PDMDEP-34335</t>
         </is>
       </c>
       <c r="M180" s="14" t="inlineStr">
         <is>
-          <t>00167140</t>
+          <t>00168072</t>
         </is>
       </c>
       <c r="N180" s="15" t="n">
-        <v>510.6</v>
-      </c>
-      <c r="O180" s="16" t="n">
-        <v>170.2</v>
+        <v>0</v>
+      </c>
+      <c r="O180" s="15" t="n">
+        <v>150</v>
       </c>
       <c r="P180" s="15" t="n">
         <v>0</v>
@@ -13395,18 +13399,18 @@
     <row r="181">
       <c r="A181" s="10" t="inlineStr">
         <is>
-          <t>PSC-1240</t>
+          <t>PSC-1270</t>
         </is>
       </c>
       <c r="B181" s="11" t="inlineStr">
         <is>
-          <t>COMMUNE DE BRANNE</t>
+          <t>COMMUNE DE CASTELNAUDARY</t>
         </is>
       </c>
       <c r="C181" s="11" t="inlineStr"/>
       <c r="D181" s="11" t="inlineStr">
         <is>
-          <t>COMMUNE DE BRANNE</t>
+          <t>COMMUNE DE CASTELNAUDARY</t>
         </is>
       </c>
       <c r="E181" s="11" t="inlineStr"/>
@@ -13423,30 +13427,30 @@
       <c r="H181" s="11" t="inlineStr"/>
       <c r="I181" s="11" t="inlineStr">
         <is>
-          <t>28/04/2026</t>
+          <t>19/05/2026</t>
         </is>
       </c>
       <c r="J181" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K181" s="11" t="n">
         <v>0</v>
       </c>
       <c r="L181" s="11" t="inlineStr">
         <is>
-          <t>PDMDEP-33167</t>
+          <t>PDMDEP-33362</t>
         </is>
       </c>
       <c r="M181" s="11" t="inlineStr">
         <is>
-          <t>00165437</t>
+          <t>00167140</t>
         </is>
       </c>
       <c r="N181" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="O181" s="12" t="n">
-        <v>100</v>
+        <v>510.6</v>
+      </c>
+      <c r="O181" s="16" t="n">
+        <v>170.2</v>
       </c>
       <c r="P181" s="12" t="n">
         <v>0</v>
@@ -13455,18 +13459,18 @@
     <row r="182">
       <c r="A182" s="13" t="inlineStr">
         <is>
-          <t>PSC-1182</t>
+          <t>PSC-1240</t>
         </is>
       </c>
       <c r="B182" s="14" t="inlineStr">
         <is>
-          <t>Commune de La Ville aux Dames</t>
+          <t>COMMUNE DE BRANNE</t>
         </is>
       </c>
       <c r="C182" s="14" t="inlineStr"/>
       <c r="D182" s="14" t="inlineStr">
         <is>
-          <t>Commune de La Ville aux Dames</t>
+          <t>COMMUNE DE BRANNE</t>
         </is>
       </c>
       <c r="E182" s="14" t="inlineStr"/>
@@ -13477,28 +13481,36 @@
       </c>
       <c r="G182" s="14" t="inlineStr">
         <is>
-          <t>Commande sans prestation</t>
+          <t>Projet</t>
         </is>
       </c>
       <c r="H182" s="14" t="inlineStr"/>
       <c r="I182" s="14" t="inlineStr">
         <is>
-          <t>10/03/2026</t>
+          <t>28/04/2026</t>
         </is>
       </c>
       <c r="J182" s="14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K182" s="14" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="L182" s="14" t="inlineStr"/>
-      <c r="M182" s="14" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="L182" s="14" t="inlineStr">
+        <is>
+          <t>PDMDEP-33167</t>
+        </is>
+      </c>
+      <c r="M182" s="14" t="inlineStr">
+        <is>
+          <t>00165437</t>
+        </is>
+      </c>
       <c r="N182" s="15" t="n">
         <v>0</v>
       </c>
       <c r="O182" s="15" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="P182" s="15" t="n">
         <v>0</v>
@@ -13507,18 +13519,18 @@
     <row r="183">
       <c r="A183" s="10" t="inlineStr">
         <is>
-          <t>PSC-1126</t>
+          <t>PSC-1182</t>
         </is>
       </c>
       <c r="B183" s="11" t="inlineStr">
         <is>
-          <t>COMMUNE DE CARRY LE ROUET</t>
+          <t>Commune de La Ville aux Dames</t>
         </is>
       </c>
       <c r="C183" s="11" t="inlineStr"/>
       <c r="D183" s="11" t="inlineStr">
         <is>
-          <t>COMMUNE DE CARRY LE ROUET</t>
+          <t>Commune de La Ville aux Dames</t>
         </is>
       </c>
       <c r="E183" s="11" t="inlineStr"/>
@@ -13535,14 +13547,14 @@
       <c r="H183" s="11" t="inlineStr"/>
       <c r="I183" s="11" t="inlineStr">
         <is>
-          <t>26/01/2026</t>
+          <t>10/03/2026</t>
         </is>
       </c>
       <c r="J183" s="11" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K183" s="11" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="L183" s="11" t="inlineStr"/>
       <c r="M183" s="11" t="inlineStr"/>
@@ -13559,18 +13571,18 @@
     <row r="184">
       <c r="A184" s="13" t="inlineStr">
         <is>
-          <t>PSC-1021</t>
+          <t>PSC-1126</t>
         </is>
       </c>
       <c r="B184" s="14" t="inlineStr">
         <is>
-          <t>MAIRIE DE MELESSE</t>
+          <t>COMMUNE DE CARRY LE ROUET</t>
         </is>
       </c>
       <c r="C184" s="14" t="inlineStr"/>
       <c r="D184" s="14" t="inlineStr">
         <is>
-          <t>MAIRIE DE MELESSE</t>
+          <t>COMMUNE DE CARRY LE ROUET</t>
         </is>
       </c>
       <c r="E184" s="14" t="inlineStr"/>
@@ -13587,14 +13599,14 @@
       <c r="H184" s="14" t="inlineStr"/>
       <c r="I184" s="14" t="inlineStr">
         <is>
-          <t>06/10/2025</t>
+          <t>26/01/2026</t>
         </is>
       </c>
       <c r="J184" s="14" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="K184" s="14" t="n">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="L184" s="14" t="inlineStr"/>
       <c r="M184" s="14" t="inlineStr"/>
@@ -13611,18 +13623,18 @@
     <row r="185">
       <c r="A185" s="10" t="inlineStr">
         <is>
-          <t>PSC-589</t>
+          <t>PSC-1021</t>
         </is>
       </c>
       <c r="B185" s="11" t="inlineStr">
         <is>
-          <t>Mairie de Venelles</t>
+          <t>MAIRIE DE MELESSE</t>
         </is>
       </c>
       <c r="C185" s="11" t="inlineStr"/>
       <c r="D185" s="11" t="inlineStr">
         <is>
-          <t>Mairie de Venelles</t>
+          <t>MAIRIE DE MELESSE</t>
         </is>
       </c>
       <c r="E185" s="11" t="inlineStr"/>
@@ -13639,11 +13651,11 @@
       <c r="H185" s="11" t="inlineStr"/>
       <c r="I185" s="11" t="inlineStr">
         <is>
-          <t>20/03/2025</t>
+          <t>06/10/2025</t>
         </is>
       </c>
       <c r="J185" s="11" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="K185" s="11" t="n">
         <v>0.5</v>
@@ -13661,31 +13673,83 @@
       </c>
     </row>
     <row r="186">
-      <c r="A186" s="17" t="inlineStr">
+      <c r="A186" s="13" t="inlineStr">
+        <is>
+          <t>PSC-589</t>
+        </is>
+      </c>
+      <c r="B186" s="14" t="inlineStr">
+        <is>
+          <t>Mairie de Venelles</t>
+        </is>
+      </c>
+      <c r="C186" s="14" t="inlineStr"/>
+      <c r="D186" s="14" t="inlineStr">
+        <is>
+          <t>Mairie de Venelles</t>
+        </is>
+      </c>
+      <c r="E186" s="14" t="inlineStr"/>
+      <c r="F186" s="14" t="inlineStr">
+        <is>
+          <t>LITTERALIS</t>
+        </is>
+      </c>
+      <c r="G186" s="14" t="inlineStr">
+        <is>
+          <t>Commande sans prestation</t>
+        </is>
+      </c>
+      <c r="H186" s="14" t="inlineStr"/>
+      <c r="I186" s="14" t="inlineStr">
+        <is>
+          <t>20/03/2025</t>
+        </is>
+      </c>
+      <c r="J186" s="14" t="n">
+        <v>16</v>
+      </c>
+      <c r="K186" s="14" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L186" s="14" t="inlineStr"/>
+      <c r="M186" s="14" t="inlineStr"/>
+      <c r="N186" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="O186" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P186" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="17" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B186" s="17" t="inlineStr"/>
-      <c r="C186" s="17" t="inlineStr"/>
-      <c r="D186" s="17" t="inlineStr"/>
-      <c r="E186" s="17" t="inlineStr"/>
-      <c r="F186" s="17" t="inlineStr"/>
-      <c r="G186" s="17" t="inlineStr"/>
-      <c r="H186" s="17" t="inlineStr"/>
-      <c r="I186" s="17" t="inlineStr"/>
-      <c r="J186" s="17" t="inlineStr"/>
-      <c r="K186" s="17" t="inlineStr"/>
-      <c r="L186" s="17" t="inlineStr"/>
-      <c r="M186" s="17" t="inlineStr"/>
-      <c r="N186" s="18" t="n">
-        <v>65939.26000000001</v>
-      </c>
-      <c r="O186" s="18" t="n">
-        <v>60144.79500000001</v>
-      </c>
-      <c r="P186" s="18" t="n">
-        <v>177.94</v>
+      <c r="B187" s="17" t="inlineStr"/>
+      <c r="C187" s="17" t="inlineStr"/>
+      <c r="D187" s="17" t="inlineStr"/>
+      <c r="E187" s="17" t="inlineStr"/>
+      <c r="F187" s="17" t="inlineStr"/>
+      <c r="G187" s="17" t="inlineStr"/>
+      <c r="H187" s="17" t="inlineStr"/>
+      <c r="I187" s="17" t="inlineStr"/>
+      <c r="J187" s="17" t="inlineStr"/>
+      <c r="K187" s="17" t="inlineStr"/>
+      <c r="L187" s="17" t="inlineStr"/>
+      <c r="M187" s="17" t="inlineStr"/>
+      <c r="N187" s="18" t="n">
+        <v>63691.76</v>
+      </c>
+      <c r="O187" s="18" t="n">
+        <v>60599.475</v>
+      </c>
+      <c r="P187" s="18" t="n">
+        <v>176.42</v>
       </c>
     </row>
   </sheetData>
@@ -13872,6 +13936,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A183" r:id="rId179"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A184" r:id="rId180"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A185" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A186" r:id="rId182"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -14899,26 +14964,26 @@
         </is>
       </c>
       <c r="B5" s="14" t="n">
-        <v>189</v>
+        <v>194.25</v>
       </c>
       <c r="C5" s="14" t="n">
-        <v>34.75</v>
+        <v>35</v>
       </c>
       <c r="D5" s="14" t="n">
         <v>3</v>
       </c>
       <c r="E5" s="14" t="n">
-        <v>226.75</v>
+        <v>232.25</v>
       </c>
       <c r="F5" s="14" t="n">
-        <v>65.5</v>
+        <v>66</v>
       </c>
       <c r="G5" s="14" t="n">
         <v>486.15</v>
       </c>
       <c r="H5" s="21" t="inlineStr">
         <is>
-          <t>46.6%</t>
+          <t>47.8%</t>
         </is>
       </c>
     </row>
@@ -14960,7 +15025,7 @@
         </is>
       </c>
       <c r="B8" s="23" t="n">
-        <v>119.83</v>
+        <v>124.83</v>
       </c>
     </row>
   </sheetData>
@@ -15045,16 +15110,16 @@
         </is>
       </c>
       <c r="B5" s="24" t="n">
-        <v>381131</v>
+        <v>383426</v>
       </c>
       <c r="C5" s="24" t="n">
-        <v>122302</v>
+        <v>123618</v>
       </c>
       <c r="D5" s="24" t="n">
-        <v>258828</v>
+        <v>259808</v>
       </c>
       <c r="E5" s="24" t="n">
-        <v>166857</v>
+        <v>167737</v>
       </c>
       <c r="F5" s="24" t="n">
         <v>22749</v>
@@ -15070,13 +15135,13 @@
         </is>
       </c>
       <c r="B6" s="25" t="n">
-        <v>174159</v>
+        <v>176649</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>68277</v>
+        <v>70667</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>105882</v>
+        <v>105982</v>
       </c>
       <c r="E6" s="25" t="n">
         <v>87486</v>
@@ -15095,16 +15160,16 @@
         </is>
       </c>
       <c r="B7" s="26" t="n">
-        <v>206972</v>
+        <v>206777</v>
       </c>
       <c r="C7" s="26" t="n">
-        <v>54026</v>
+        <v>52951</v>
       </c>
       <c r="D7" s="26" t="n">
-        <v>152946</v>
+        <v>153826</v>
       </c>
       <c r="E7" s="26" t="n">
-        <v>79371</v>
+        <v>80251</v>
       </c>
       <c r="F7" s="26" t="n">
         <v>10557</v>
@@ -15124,7 +15189,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -15148,7 +15213,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Épics créées ce mois — 18 commande(s)</t>
+          <t>Épics créées ce mois — 17 commande(s)</t>
         </is>
       </c>
     </row>
@@ -15428,34 +15493,34 @@
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>PDMDEP-34566</t>
+          <t>PDMDEP-34589</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>PDMDEP-34559</t>
+          <t>PDMDEP-34580</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>15/07/2026</t>
+          <t>16/07/2026</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
+          <t>COMMUNE DE RIEZ</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="inlineStr">
+        <is>
+          <t>GEODP</t>
+        </is>
+      </c>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
           <t>Migration</t>
         </is>
       </c>
-      <c r="E10" s="11" t="inlineStr">
-        <is>
-          <t>GEODP</t>
-        </is>
-      </c>
-      <c r="F10" s="11" t="inlineStr">
-        <is>
-          <t>Migration</t>
-        </is>
-      </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
           <t>Services</t>
@@ -15463,32 +15528,32 @@
       </c>
       <c r="H10" s="11" t="inlineStr">
         <is>
-          <t>00154892</t>
+          <t>00176128</t>
         </is>
       </c>
       <c r="I10" s="26" t="n">
-        <v>5000</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-34589</t>
+          <t>PDMDEP-34420</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-34580</t>
+          <t>PDMDEP-34411</t>
         </is>
       </c>
       <c r="C11" s="14" t="inlineStr">
         <is>
-          <t>16/07/2026</t>
+          <t>02/07/2026</t>
         </is>
       </c>
       <c r="D11" s="14" t="inlineStr">
         <is>
-          <t>COMMUNE DE RIEZ</t>
+          <t>MAIRIE DE MAIZIERES LES METZ</t>
         </is>
       </c>
       <c r="E11" s="14" t="inlineStr">
@@ -15508,32 +15573,32 @@
       </c>
       <c r="H11" s="14" t="inlineStr">
         <is>
-          <t>00176128</t>
+          <t>00172317</t>
         </is>
       </c>
       <c r="I11" s="25" t="n">
-        <v>1300</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>PDMDEP-34420</t>
+          <t>PDMDEP-34396</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>PDMDEP-34411</t>
+          <t>PDMDEP-34390</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>02/07/2026</t>
+          <t>01/07/2026</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>MAIRIE DE MAIZIERES LES METZ</t>
+          <t>Commune Le THOR</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
@@ -15543,7 +15608,7 @@
       </c>
       <c r="F12" s="11" t="inlineStr">
         <is>
-          <t>Migration</t>
+          <t>Vente additionnelle</t>
         </is>
       </c>
       <c r="G12" s="11" t="inlineStr">
@@ -15553,32 +15618,32 @@
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>00172317</t>
+          <t>00171793</t>
         </is>
       </c>
       <c r="I12" s="26" t="n">
-        <v>2035</v>
+        <v>250</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-34396</t>
+          <t>PDMDEP-34666</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-34390</t>
+          <t>PDMDEP-34659</t>
         </is>
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
-          <t>01/07/2026</t>
+          <t>22/07/2026</t>
         </is>
       </c>
       <c r="D13" s="14" t="inlineStr">
         <is>
-          <t>Commune Le THOR</t>
+          <t>Commune des Ponts de Ce</t>
         </is>
       </c>
       <c r="E13" s="14" t="inlineStr">
@@ -15588,7 +15653,7 @@
       </c>
       <c r="F13" s="14" t="inlineStr">
         <is>
-          <t>Vente additionnelle</t>
+          <t>Migration</t>
         </is>
       </c>
       <c r="G13" s="14" t="inlineStr">
@@ -15598,22 +15663,22 @@
       </c>
       <c r="H13" s="14" t="inlineStr">
         <is>
-          <t>00171793</t>
+          <t>00176614</t>
         </is>
       </c>
       <c r="I13" s="25" t="n">
-        <v>250</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>PDMDEP-34666</t>
+          <t>PDMDEP-34683</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>PDMDEP-34659</t>
+          <t>PDMDEP-34676</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
@@ -15647,18 +15712,18 @@
         </is>
       </c>
       <c r="I14" s="26" t="n">
-        <v>2000</v>
+        <v>2150</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-34683</t>
+          <t>PDMDEP-34701</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-34676</t>
+          <t>PDMDEP-34694</t>
         </is>
       </c>
       <c r="C15" s="14" t="inlineStr">
@@ -15668,7 +15733,7 @@
       </c>
       <c r="D15" s="14" t="inlineStr">
         <is>
-          <t>Commune des Ponts de Ce</t>
+          <t>Commune du Tampon</t>
         </is>
       </c>
       <c r="E15" s="14" t="inlineStr">
@@ -15688,32 +15753,32 @@
       </c>
       <c r="H15" s="14" t="inlineStr">
         <is>
-          <t>00176614</t>
+          <t>00176675</t>
         </is>
       </c>
       <c r="I15" s="25" t="n">
-        <v>2150</v>
+        <v>3947.5</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>PDMDEP-34701</t>
+          <t>PDMDEP-34768</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>PDMDEP-34694</t>
+          <t>PDMDEP-34761</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>22/07/2026</t>
+          <t>28/07/2026</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Commune du Tampon</t>
+          <t>COMMUNE DU PUY EN VELAY</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
@@ -15733,32 +15798,32 @@
       </c>
       <c r="H16" s="11" t="inlineStr">
         <is>
-          <t>00176675</t>
+          <t>00177029</t>
         </is>
       </c>
       <c r="I16" s="26" t="n">
-        <v>3947.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-34768</t>
+          <t>PDMDEP-34640</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-34761</t>
+          <t>PDMDEP-34631</t>
         </is>
       </c>
       <c r="C17" s="14" t="inlineStr">
         <is>
-          <t>28/07/2026</t>
+          <t>21/07/2026</t>
         </is>
       </c>
       <c r="D17" s="14" t="inlineStr">
         <is>
-          <t>COMMUNE DU PUY EN VELAY</t>
+          <t>COMMUNE DE SAINT-HILAIRE-DE-RIEZ</t>
         </is>
       </c>
       <c r="E17" s="14" t="inlineStr">
@@ -15768,7 +15833,7 @@
       </c>
       <c r="F17" s="14" t="inlineStr">
         <is>
-          <t>Migration</t>
+          <t>Nouveau déploiement</t>
         </is>
       </c>
       <c r="G17" s="14" t="inlineStr">
@@ -15778,22 +15843,22 @@
       </c>
       <c r="H17" s="14" t="inlineStr">
         <is>
-          <t>00177029</t>
+          <t>00176477</t>
         </is>
       </c>
       <c r="I17" s="25" t="n">
-        <v>0</v>
+        <v>2250</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>PDMDEP-34640</t>
+          <t>PDMDEP-34654</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>PDMDEP-34631</t>
+          <t>PDMDEP-34650</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
@@ -15803,17 +15868,17 @@
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>COMMUNE DE SAINT-HILAIRE-DE-RIEZ</t>
+          <t>DEPARTEMENT DE L AIN (CD 01)</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>GEODP</t>
+          <t>LITTERALIS</t>
         </is>
       </c>
       <c r="F18" s="11" t="inlineStr">
         <is>
-          <t>Nouveau déploiement</t>
+          <t>Vente additionnelle</t>
         </is>
       </c>
       <c r="G18" s="11" t="inlineStr">
@@ -15823,32 +15888,32 @@
       </c>
       <c r="H18" s="11" t="inlineStr">
         <is>
-          <t>00176477</t>
+          <t>00176582</t>
         </is>
       </c>
       <c r="I18" s="26" t="n">
-        <v>2250</v>
+        <v>495</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-34654</t>
+          <t>PDMDEP-34499</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-34650</t>
+          <t>PDMDEP-34495</t>
         </is>
       </c>
       <c r="C19" s="14" t="inlineStr">
         <is>
-          <t>21/07/2026</t>
+          <t>07/07/2026</t>
         </is>
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
-          <t>DEPARTEMENT DE L AIN (CD 01)</t>
+          <t>COMMUNE DE CLICHY</t>
         </is>
       </c>
       <c r="E19" s="14" t="inlineStr">
@@ -15868,32 +15933,32 @@
       </c>
       <c r="H19" s="14" t="inlineStr">
         <is>
-          <t>00176582</t>
+          <t>00172678</t>
         </is>
       </c>
       <c r="I19" s="25" t="n">
-        <v>495</v>
+        <v>4300</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="11" t="inlineStr">
         <is>
-          <t>PDMDEP-34499</t>
+          <t>PDMDEP-34722</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>PDMDEP-34495</t>
+          <t>PDMDEP-34718</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>07/07/2026</t>
+          <t>24/07/2026</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>COMMUNE DE CLICHY</t>
+          <t>VILLE DE VILLEURBANNE</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
@@ -15913,32 +15978,32 @@
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>00172678</t>
+          <t>00176875</t>
         </is>
       </c>
       <c r="I20" s="26" t="n">
-        <v>4300</v>
+        <v>2800</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-34722</t>
+          <t>PDMDEP-34778</t>
         </is>
       </c>
       <c r="B21" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-34718</t>
+          <t>PSC-1315</t>
         </is>
       </c>
       <c r="C21" s="14" t="inlineStr">
         <is>
-          <t>24/07/2026</t>
+          <t>08/07/2026</t>
         </is>
       </c>
       <c r="D21" s="14" t="inlineStr">
         <is>
-          <t>VILLE DE VILLEURBANNE</t>
+          <t>Rang-du-Fliers</t>
         </is>
       </c>
       <c r="E21" s="14" t="inlineStr">
@@ -15946,62 +16011,38 @@
           <t>LITTERALIS</t>
         </is>
       </c>
-      <c r="F21" s="14" t="inlineStr">
-        <is>
-          <t>Vente additionnelle</t>
-        </is>
-      </c>
-      <c r="G21" s="14" t="inlineStr">
-        <is>
-          <t>Services</t>
-        </is>
-      </c>
-      <c r="H21" s="14" t="inlineStr">
-        <is>
-          <t>00176875</t>
-        </is>
-      </c>
+      <c r="F21" s="14" t="inlineStr"/>
+      <c r="G21" s="14" t="inlineStr"/>
+      <c r="H21" s="14" t="inlineStr"/>
       <c r="I21" s="25" t="n">
-        <v>2800</v>
+        <v>500</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="11" t="inlineStr">
-        <is>
-          <t>PDMDEP-34778</t>
-        </is>
-      </c>
-      <c r="B22" s="11" t="inlineStr">
-        <is>
-          <t>PSC-1315</t>
-        </is>
-      </c>
-      <c r="C22" s="11" t="inlineStr">
-        <is>
-          <t>08/07/2026</t>
-        </is>
-      </c>
-      <c r="D22" s="11" t="inlineStr">
-        <is>
-          <t>Rang-du-Fliers</t>
-        </is>
-      </c>
-      <c r="E22" s="11" t="inlineStr">
-        <is>
-          <t>LITTERALIS</t>
-        </is>
-      </c>
-      <c r="F22" s="11" t="inlineStr"/>
-      <c r="G22" s="11" t="inlineStr"/>
-      <c r="H22" s="11" t="inlineStr"/>
-      <c r="I22" s="26" t="n">
-        <v>500</v>
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="n"/>
+      <c r="C22" s="17" t="n"/>
+      <c r="D22" s="17" t="n"/>
+      <c r="E22" s="17" t="n"/>
+      <c r="F22" s="17" t="n"/>
+      <c r="G22" s="17" t="n"/>
+      <c r="H22" s="17" t="inlineStr">
+        <is>
+          <t>17 commande(s)</t>
+        </is>
+      </c>
+      <c r="I22" s="24" t="n">
+        <v>31052</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="17" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>dont Littéralis</t>
         </is>
       </c>
       <c r="B23" s="17" t="n"/>
@@ -16012,17 +16053,17 @@
       <c r="G23" s="17" t="n"/>
       <c r="H23" s="17" t="inlineStr">
         <is>
-          <t>18 commande(s)</t>
+          <t>4 commande(s)</t>
         </is>
       </c>
       <c r="I23" s="24" t="n">
-        <v>36052</v>
+        <v>8095</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="17" t="inlineStr">
         <is>
-          <t>dont Littéralis</t>
+          <t>dont GEODP</t>
         </is>
       </c>
       <c r="B24" s="17" t="n"/>
@@ -16033,32 +16074,11 @@
       <c r="G24" s="17" t="n"/>
       <c r="H24" s="17" t="inlineStr">
         <is>
-          <t>4 commande(s)</t>
+          <t>13 commande(s)</t>
         </is>
       </c>
       <c r="I24" s="24" t="n">
-        <v>8095</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="17" t="inlineStr">
-        <is>
-          <t>dont GEODP</t>
-        </is>
-      </c>
-      <c r="B25" s="17" t="n"/>
-      <c r="C25" s="17" t="n"/>
-      <c r="D25" s="17" t="n"/>
-      <c r="E25" s="17" t="n"/>
-      <c r="F25" s="17" t="n"/>
-      <c r="G25" s="17" t="n"/>
-      <c r="H25" s="17" t="inlineStr">
-        <is>
-          <t>14 commande(s)</t>
-        </is>
-      </c>
-      <c r="I25" s="24" t="n">
-        <v>27958</v>
+        <v>22958</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MAJ pipeline 2026-07-29 08:52
</commit_message>
<xml_diff>
--- a/jira_export_2026-07-29.xlsx
+++ b/jira_export_2026-07-29.xlsx
@@ -723,7 +723,7 @@
     <row r="7" ht="26" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>60,599 €</t>
+          <t>61,679 €</t>
         </is>
       </c>
       <c r="B7" s="7" t="n"/>
@@ -737,7 +737,7 @@
       <c r="F7" s="7" t="n"/>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>63.8%</t>
+          <t>64.9%</t>
         </is>
       </c>
       <c r="H7" s="7" t="n"/>
@@ -770,7 +770,7 @@
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>38,293 €</t>
+          <t>39,373 €</t>
         </is>
       </c>
       <c r="E11" s="7" t="n"/>
@@ -818,7 +818,7 @@
     <row r="16" ht="26" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>558 h</t>
+          <t>559 h</t>
         </is>
       </c>
       <c r="B16" s="7" t="n"/>
@@ -889,7 +889,7 @@
     <row r="25" ht="26" customHeight="1">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B25" s="7" t="n"/>
@@ -903,7 +903,7 @@
       <c r="F25" s="7" t="n"/>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>258</t>
+          <t>255</t>
         </is>
       </c>
       <c r="H25" s="7" t="n"/>
@@ -7193,10 +7193,10 @@
         </is>
       </c>
       <c r="N90" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="O90" s="15" t="n">
         <v>45</v>
-      </c>
-      <c r="O90" s="16" t="n">
-        <v>0</v>
       </c>
       <c r="P90" s="15" t="n">
         <v>0</v>
@@ -10525,10 +10525,10 @@
         </is>
       </c>
       <c r="N137" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O137" s="12" t="n">
         <v>964.1</v>
-      </c>
-      <c r="O137" s="16" t="n">
-        <v>0</v>
       </c>
       <c r="P137" s="12" t="n">
         <v>0</v>
@@ -10595,10 +10595,10 @@
         </is>
       </c>
       <c r="N138" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="O138" s="15" t="n">
         <v>140.4</v>
-      </c>
-      <c r="O138" s="16" t="n">
-        <v>70.2</v>
       </c>
       <c r="P138" s="15" t="n">
         <v>0</v>
@@ -13743,13 +13743,13 @@
       <c r="L187" s="17" t="inlineStr"/>
       <c r="M187" s="17" t="inlineStr"/>
       <c r="N187" s="18" t="n">
-        <v>63691.76</v>
+        <v>62542.26</v>
       </c>
       <c r="O187" s="18" t="n">
-        <v>60599.475</v>
+        <v>61678.775</v>
       </c>
       <c r="P187" s="18" t="n">
-        <v>176.42</v>
+        <v>179.56</v>
       </c>
     </row>
   </sheetData>
@@ -15025,7 +15025,7 @@
         </is>
       </c>
       <c r="B8" s="23" t="n">
-        <v>124.83</v>
+        <v>125.33</v>
       </c>
     </row>
   </sheetData>
@@ -15110,16 +15110,16 @@
         </is>
       </c>
       <c r="B5" s="24" t="n">
-        <v>383426</v>
+        <v>382277</v>
       </c>
       <c r="C5" s="24" t="n">
-        <v>123618</v>
+        <v>123573</v>
       </c>
       <c r="D5" s="24" t="n">
-        <v>259808</v>
+        <v>258704</v>
       </c>
       <c r="E5" s="24" t="n">
-        <v>167737</v>
+        <v>166632</v>
       </c>
       <c r="F5" s="24" t="n">
         <v>22749</v>
@@ -15160,16 +15160,16 @@
         </is>
       </c>
       <c r="B7" s="26" t="n">
-        <v>206777</v>
+        <v>205627</v>
       </c>
       <c r="C7" s="26" t="n">
-        <v>52951</v>
+        <v>52906</v>
       </c>
       <c r="D7" s="26" t="n">
-        <v>153826</v>
+        <v>152722</v>
       </c>
       <c r="E7" s="26" t="n">
-        <v>80251</v>
+        <v>79146</v>
       </c>
       <c r="F7" s="26" t="n">
         <v>10557</v>
@@ -15189,7 +15189,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -15213,7 +15213,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Épics créées ce mois — 17 commande(s)</t>
+          <t>Épics créées ce mois — 18 commande(s)</t>
         </is>
       </c>
     </row>
@@ -15268,22 +15268,22 @@
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-34621</t>
+          <t>PDMDEP-34791</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-34613</t>
+          <t>PDMDEP-34782</t>
         </is>
       </c>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>20/07/2026</t>
+          <t>29/07/2026</t>
         </is>
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
-          <t>COMMUNE DE FORT-DE-FRANCE</t>
+          <t>MAIRIE DE SAINT-ISMIER</t>
         </is>
       </c>
       <c r="E5" s="14" t="inlineStr">
@@ -15293,7 +15293,7 @@
       </c>
       <c r="F5" s="14" t="inlineStr">
         <is>
-          <t>Vente additionnelle</t>
+          <t>Nouveau déploiement</t>
         </is>
       </c>
       <c r="G5" s="14" t="inlineStr">
@@ -15303,11 +15303,11 @@
       </c>
       <c r="H5" s="14" t="inlineStr">
         <is>
-          <t>00176431</t>
+          <t>00177122</t>
         </is>
       </c>
       <c r="I5" s="25" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -15538,22 +15538,22 @@
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-34420</t>
+          <t>PDMDEP-34621</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-34411</t>
+          <t>PDMDEP-34613</t>
         </is>
       </c>
       <c r="C11" s="14" t="inlineStr">
         <is>
-          <t>02/07/2026</t>
+          <t>20/07/2026</t>
         </is>
       </c>
       <c r="D11" s="14" t="inlineStr">
         <is>
-          <t>MAIRIE DE MAIZIERES LES METZ</t>
+          <t>COMMUNE DE FORT-DE-FRANCE</t>
         </is>
       </c>
       <c r="E11" s="14" t="inlineStr">
@@ -15563,7 +15563,7 @@
       </c>
       <c r="F11" s="14" t="inlineStr">
         <is>
-          <t>Migration</t>
+          <t>Vente additionnelle</t>
         </is>
       </c>
       <c r="G11" s="14" t="inlineStr">
@@ -15573,32 +15573,32 @@
       </c>
       <c r="H11" s="14" t="inlineStr">
         <is>
-          <t>00172317</t>
+          <t>00176431</t>
         </is>
       </c>
       <c r="I11" s="25" t="n">
-        <v>2035</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>PDMDEP-34396</t>
+          <t>PDMDEP-34420</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>PDMDEP-34390</t>
+          <t>PDMDEP-34411</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>01/07/2026</t>
+          <t>02/07/2026</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Commune Le THOR</t>
+          <t>MAIRIE DE MAIZIERES LES METZ</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
@@ -15608,7 +15608,7 @@
       </c>
       <c r="F12" s="11" t="inlineStr">
         <is>
-          <t>Vente additionnelle</t>
+          <t>Migration</t>
         </is>
       </c>
       <c r="G12" s="11" t="inlineStr">
@@ -15618,32 +15618,32 @@
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>00171793</t>
+          <t>00172317</t>
         </is>
       </c>
       <c r="I12" s="26" t="n">
-        <v>250</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-34666</t>
+          <t>PDMDEP-34640</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-34659</t>
+          <t>PDMDEP-34631</t>
         </is>
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
-          <t>22/07/2026</t>
+          <t>21/07/2026</t>
         </is>
       </c>
       <c r="D13" s="14" t="inlineStr">
         <is>
-          <t>Commune des Ponts de Ce</t>
+          <t>COMMUNE DE SAINT-HILAIRE-DE-RIEZ</t>
         </is>
       </c>
       <c r="E13" s="14" t="inlineStr">
@@ -15653,7 +15653,7 @@
       </c>
       <c r="F13" s="14" t="inlineStr">
         <is>
-          <t>Migration</t>
+          <t>Nouveau déploiement</t>
         </is>
       </c>
       <c r="G13" s="14" t="inlineStr">
@@ -15663,22 +15663,22 @@
       </c>
       <c r="H13" s="14" t="inlineStr">
         <is>
-          <t>00176614</t>
+          <t>00176477</t>
         </is>
       </c>
       <c r="I13" s="25" t="n">
-        <v>2000</v>
+        <v>2250</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>PDMDEP-34683</t>
+          <t>PDMDEP-34666</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>PDMDEP-34676</t>
+          <t>PDMDEP-34659</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
@@ -15712,18 +15712,18 @@
         </is>
       </c>
       <c r="I14" s="26" t="n">
-        <v>2150</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-34701</t>
+          <t>PDMDEP-34683</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-34694</t>
+          <t>PDMDEP-34676</t>
         </is>
       </c>
       <c r="C15" s="14" t="inlineStr">
@@ -15733,7 +15733,7 @@
       </c>
       <c r="D15" s="14" t="inlineStr">
         <is>
-          <t>Commune du Tampon</t>
+          <t>Commune des Ponts de Ce</t>
         </is>
       </c>
       <c r="E15" s="14" t="inlineStr">
@@ -15753,32 +15753,32 @@
       </c>
       <c r="H15" s="14" t="inlineStr">
         <is>
-          <t>00176675</t>
+          <t>00176614</t>
         </is>
       </c>
       <c r="I15" s="25" t="n">
-        <v>3947.5</v>
+        <v>2150</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>PDMDEP-34768</t>
+          <t>PDMDEP-34701</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>PDMDEP-34761</t>
+          <t>PDMDEP-34694</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>28/07/2026</t>
+          <t>22/07/2026</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>COMMUNE DU PUY EN VELAY</t>
+          <t>Commune du Tampon</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
@@ -15798,32 +15798,32 @@
       </c>
       <c r="H16" s="11" t="inlineStr">
         <is>
-          <t>00177029</t>
+          <t>00176675</t>
         </is>
       </c>
       <c r="I16" s="26" t="n">
-        <v>0</v>
+        <v>3947.5</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-34640</t>
+          <t>PDMDEP-34768</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-34631</t>
+          <t>PDMDEP-34761</t>
         </is>
       </c>
       <c r="C17" s="14" t="inlineStr">
         <is>
-          <t>21/07/2026</t>
+          <t>28/07/2026</t>
         </is>
       </c>
       <c r="D17" s="14" t="inlineStr">
         <is>
-          <t>COMMUNE DE SAINT-HILAIRE-DE-RIEZ</t>
+          <t>COMMUNE DU PUY EN VELAY</t>
         </is>
       </c>
       <c r="E17" s="14" t="inlineStr">
@@ -15833,7 +15833,7 @@
       </c>
       <c r="F17" s="14" t="inlineStr">
         <is>
-          <t>Nouveau déploiement</t>
+          <t>Migration</t>
         </is>
       </c>
       <c r="G17" s="14" t="inlineStr">
@@ -15843,37 +15843,37 @@
       </c>
       <c r="H17" s="14" t="inlineStr">
         <is>
-          <t>00176477</t>
+          <t>00177029</t>
         </is>
       </c>
       <c r="I17" s="25" t="n">
-        <v>2250</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>PDMDEP-34654</t>
+          <t>PDMDEP-34396</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>PDMDEP-34650</t>
+          <t>PDMDEP-34390</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>21/07/2026</t>
+          <t>01/07/2026</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>DEPARTEMENT DE L AIN (CD 01)</t>
+          <t>Commune Le THOR</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>LITTERALIS</t>
+          <t>GEODP</t>
         </is>
       </c>
       <c r="F18" s="11" t="inlineStr">
@@ -15888,32 +15888,32 @@
       </c>
       <c r="H18" s="11" t="inlineStr">
         <is>
-          <t>00176582</t>
+          <t>00171793</t>
         </is>
       </c>
       <c r="I18" s="26" t="n">
-        <v>495</v>
+        <v>250</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-34499</t>
+          <t>PDMDEP-34722</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-34495</t>
+          <t>PDMDEP-34718</t>
         </is>
       </c>
       <c r="C19" s="14" t="inlineStr">
         <is>
-          <t>07/07/2026</t>
+          <t>24/07/2026</t>
         </is>
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
-          <t>COMMUNE DE CLICHY</t>
+          <t>VILLE DE VILLEURBANNE</t>
         </is>
       </c>
       <c r="E19" s="14" t="inlineStr">
@@ -15933,32 +15933,32 @@
       </c>
       <c r="H19" s="14" t="inlineStr">
         <is>
-          <t>00172678</t>
+          <t>00176875</t>
         </is>
       </c>
       <c r="I19" s="25" t="n">
-        <v>4300</v>
+        <v>2800</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="11" t="inlineStr">
         <is>
-          <t>PDMDEP-34722</t>
+          <t>PDMDEP-34499</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>PDMDEP-34718</t>
+          <t>PDMDEP-34495</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>24/07/2026</t>
+          <t>07/07/2026</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>VILLE DE VILLEURBANNE</t>
+          <t>COMMUNE DE CLICHY</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
@@ -15978,11 +15978,11 @@
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>00176875</t>
+          <t>00172678</t>
         </is>
       </c>
       <c r="I20" s="26" t="n">
-        <v>2800</v>
+        <v>4300</v>
       </c>
     </row>
     <row r="21">
@@ -16019,30 +16019,54 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="17" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B22" s="17" t="n"/>
-      <c r="C22" s="17" t="n"/>
-      <c r="D22" s="17" t="n"/>
-      <c r="E22" s="17" t="n"/>
-      <c r="F22" s="17" t="n"/>
-      <c r="G22" s="17" t="n"/>
-      <c r="H22" s="17" t="inlineStr">
-        <is>
-          <t>17 commande(s)</t>
-        </is>
-      </c>
-      <c r="I22" s="24" t="n">
-        <v>31052</v>
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>PDMDEP-34654</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>PDMDEP-34650</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>21/07/2026</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>DEPARTEMENT DE L AIN (CD 01)</t>
+        </is>
+      </c>
+      <c r="E22" s="11" t="inlineStr">
+        <is>
+          <t>LITTERALIS</t>
+        </is>
+      </c>
+      <c r="F22" s="11" t="inlineStr">
+        <is>
+          <t>Vente additionnelle</t>
+        </is>
+      </c>
+      <c r="G22" s="11" t="inlineStr">
+        <is>
+          <t>Services</t>
+        </is>
+      </c>
+      <c r="H22" s="11" t="inlineStr">
+        <is>
+          <t>00176582</t>
+        </is>
+      </c>
+      <c r="I22" s="26" t="n">
+        <v>495</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="17" t="inlineStr">
         <is>
-          <t>dont Littéralis</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="B23" s="17" t="n"/>
@@ -16053,17 +16077,17 @@
       <c r="G23" s="17" t="n"/>
       <c r="H23" s="17" t="inlineStr">
         <is>
-          <t>4 commande(s)</t>
+          <t>18 commande(s)</t>
         </is>
       </c>
       <c r="I23" s="24" t="n">
-        <v>8095</v>
+        <v>31052</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="17" t="inlineStr">
         <is>
-          <t>dont GEODP</t>
+          <t>dont Littéralis</t>
         </is>
       </c>
       <c r="B24" s="17" t="n"/>
@@ -16074,10 +16098,31 @@
       <c r="G24" s="17" t="n"/>
       <c r="H24" s="17" t="inlineStr">
         <is>
-          <t>13 commande(s)</t>
+          <t>4 commande(s)</t>
         </is>
       </c>
       <c r="I24" s="24" t="n">
+        <v>8095</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="17" t="inlineStr">
+        <is>
+          <t>dont GEODP</t>
+        </is>
+      </c>
+      <c r="B25" s="17" t="n"/>
+      <c r="C25" s="17" t="n"/>
+      <c r="D25" s="17" t="n"/>
+      <c r="E25" s="17" t="n"/>
+      <c r="F25" s="17" t="n"/>
+      <c r="G25" s="17" t="n"/>
+      <c r="H25" s="17" t="inlineStr">
+        <is>
+          <t>14 commande(s)</t>
+        </is>
+      </c>
+      <c r="I25" s="24" t="n">
         <v>22958</v>
       </c>
     </row>
@@ -16092,7 +16137,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="41" customWidth="1" min="1" max="1"/>
@@ -16113,7 +16158,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>13 clôture(s) : 11 projet(s), 2 rework</t>
+          <t>17 clôture(s) : 15 projet(s), 2 rework</t>
         </is>
       </c>
     </row>
@@ -16153,17 +16198,17 @@
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-30241</t>
+          <t>PDMDEP-23484</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>[MOLSHEIM] - Migration GEODP 1 vers GEODP 2 (Placier)</t>
+          <t>METROPOLE TOULON- AJOUT LIEU DE NAISSANCE DANS FILIEN</t>
         </is>
       </c>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>MOLSHEIM</t>
+          <t>METROPOLE TOULON-PROVENCE-MEDITERRANEE</t>
         </is>
       </c>
       <c r="D5" s="14" t="inlineStr">
@@ -16177,23 +16222,23 @@
         </is>
       </c>
       <c r="F5" s="14" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>PDMDEP-32331</t>
+          <t>PDMDEP-23486</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">[COMMUNE DE CHALONS EN CHAMPAGNE] - Migration GEODP Placier </t>
+          <t>METROPOLE TOULON- AJOUT BALISE FILIEN</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>COMMUNE DE CHALONS EN CHAMPAGNE</t>
+          <t>METROPOLE TOULON-PROVENCE-MEDITERRANEE</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
@@ -16207,23 +16252,23 @@
         </is>
       </c>
       <c r="F6" s="11" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-32860</t>
+          <t>PDMDEP-30241</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>[COMMUNE DE LE LUC EN PROVENCE] - MIGRATION SIMPLE GEODP PLA</t>
+          <t>[MOLSHEIM] - Migration GEODP 1 vers GEODP 2 (Placier)</t>
         </is>
       </c>
       <c r="C7" s="14" t="inlineStr">
         <is>
-          <t>COMMUNE DE LE LUC EN PROVENCE</t>
+          <t>MOLSHEIM</t>
         </is>
       </c>
       <c r="D7" s="14" t="inlineStr">
@@ -16237,23 +16282,23 @@
         </is>
       </c>
       <c r="F7" s="14" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>PDMDEP-33239</t>
+          <t>PDMDEP-31938</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>[MAIRIE DE LODEVE] - Migracier activité Placier vers Geodp V</t>
+          <t xml:space="preserve">METROPOLE TOULON- GeODP tous modules - intégration en masse </t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>MAIRIE DE LODEVE</t>
+          <t>METROPOLE TOULON-PROVENCE-MEDITERRANEE</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
@@ -16267,28 +16312,28 @@
         </is>
       </c>
       <c r="F8" s="11" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-20907</t>
+          <t>PDMDEP-32331</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>[Saint-Pierre (Réunion)] Accompagnement modélisation AME Lit</t>
+          <t xml:space="preserve">[COMMUNE DE CHALONS EN CHAMPAGNE] - Migration GEODP Placier </t>
         </is>
       </c>
       <c r="C9" s="14" t="inlineStr">
         <is>
-          <t>SAINT PIERRE (LA REUNION)</t>
+          <t>COMMUNE DE CHALONS EN CHAMPAGNE</t>
         </is>
       </c>
       <c r="D9" s="14" t="inlineStr">
         <is>
-          <t>LITTERALIS</t>
+          <t>GEODP</t>
         </is>
       </c>
       <c r="E9" s="14" t="inlineStr">
@@ -16297,28 +16342,28 @@
         </is>
       </c>
       <c r="F9" s="14" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>PDMDEP-21544</t>
+          <t>PDMDEP-32860</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>[La Ciotat] Accompagnement modélisation Littéralis Expert</t>
+          <t>[COMMUNE DE LE LUC EN PROVENCE] - MIGRATION SIMPLE GEODP PLA</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>LA CIOTAT</t>
+          <t>COMMUNE DE LE LUC EN PROVENCE</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>LITTERALIS</t>
+          <t>GEODP</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
@@ -16327,28 +16372,28 @@
         </is>
       </c>
       <c r="F10" s="11" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-26825</t>
+          <t>PDMDEP-33239</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>[COLOMBES] - Litteralis Vision &amp; Publi</t>
+          <t>[MAIRIE DE LODEVE] - Migracier activité Placier vers Geodp V</t>
         </is>
       </c>
       <c r="C11" s="14" t="inlineStr">
         <is>
-          <t>VILLE DE COLOMBES - DSIO</t>
+          <t>MAIRIE DE LODEVE</t>
         </is>
       </c>
       <c r="D11" s="14" t="inlineStr">
         <is>
-          <t>LITTERALIS</t>
+          <t>GEODP</t>
         </is>
       </c>
       <c r="E11" s="14" t="inlineStr">
@@ -16357,28 +16402,28 @@
         </is>
       </c>
       <c r="F11" s="14" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>PDMDEP-31947</t>
+          <t>PDMDEP-33553</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>[DEPARTEMENT DE LA MOSELLE (CD 57)] - SSO/LDAP</t>
+          <t>[METROPOLE TOULON-PROVENCE-MEDITERRANEE] - MM - Up - GeODP -</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>DEPARTEMENT DE LA MOSELLE (CD 57)</t>
+          <t>METROPOLE TOULON-PROVENCE-MEDITERRANEE</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>LITTERALIS</t>
+          <t>GEODP</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
@@ -16387,23 +16432,23 @@
         </is>
       </c>
       <c r="F12" s="11" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-32552</t>
+          <t>PDMDEP-20907</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>[CHALON SUR SAONE] - Littéralis - Intégration et paramétrage</t>
+          <t>[Saint-Pierre (Réunion)] Accompagnement modélisation AME Lit</t>
         </is>
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
-          <t>VILLE DE CHALON SUR SAONE</t>
+          <t>SAINT PIERRE (LA REUNION)</t>
         </is>
       </c>
       <c r="D13" s="14" t="inlineStr">
@@ -16417,23 +16462,23 @@
         </is>
       </c>
       <c r="F13" s="14" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>PDMDEP-33720</t>
+          <t>PDMDEP-21544</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>[COMMUNE DE LEVALLOIS PERRET] - PRESTA PURGE DES ACTES EN UR</t>
+          <t>[La Ciotat] Accompagnement modélisation Littéralis Expert</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>COMMUNE DE LEVALLOIS PERRET</t>
+          <t>LA CIOTAT</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -16447,125 +16492,245 @@
         </is>
       </c>
       <c r="F14" s="11" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="14" t="inlineStr">
         <is>
+          <t>PDMDEP-26825</t>
+        </is>
+      </c>
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>[COLOMBES] - Litteralis Vision &amp; Publi</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="inlineStr">
+        <is>
+          <t>VILLE DE COLOMBES - DSIO</t>
+        </is>
+      </c>
+      <c r="D15" s="14" t="inlineStr">
+        <is>
+          <t>LITTERALIS</t>
+        </is>
+      </c>
+      <c r="E15" s="14" t="inlineStr">
+        <is>
+          <t>Projet</t>
+        </is>
+      </c>
+      <c r="F15" s="14" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>PDMDEP-31947</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>[DEPARTEMENT DE LA MOSELLE (CD 57)] - SSO/LDAP</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>DEPARTEMENT DE LA MOSELLE (CD 57)</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>LITTERALIS</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="inlineStr">
+        <is>
+          <t>Projet</t>
+        </is>
+      </c>
+      <c r="F16" s="11" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>PDMDEP-32552</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>[CHALON SUR SAONE] - Littéralis - Intégration et paramétrage</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr">
+        <is>
+          <t>VILLE DE CHALON SUR SAONE</t>
+        </is>
+      </c>
+      <c r="D17" s="14" t="inlineStr">
+        <is>
+          <t>LITTERALIS</t>
+        </is>
+      </c>
+      <c r="E17" s="14" t="inlineStr">
+        <is>
+          <t>Projet</t>
+        </is>
+      </c>
+      <c r="F17" s="14" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>PDMDEP-33720</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>[COMMUNE DE LEVALLOIS PERRET] - PRESTA PURGE DES ACTES EN UR</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>COMMUNE DE LEVALLOIS PERRET</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>LITTERALIS</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>Projet</t>
+        </is>
+      </c>
+      <c r="F18" s="11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
           <t>PDMDEP-33804</t>
         </is>
       </c>
-      <c r="B15" s="14" t="inlineStr">
+      <c r="B19" s="14" t="inlineStr">
         <is>
           <t>[CD 73)] - Purge arrêtés temporaires</t>
         </is>
       </c>
-      <c r="C15" s="14" t="inlineStr">
+      <c r="C19" s="14" t="inlineStr">
         <is>
           <t>CONSEIL DEPARTEMENTAL DE LA SAVOIE (CD 73)</t>
         </is>
       </c>
-      <c r="D15" s="14" t="inlineStr">
+      <c r="D19" s="14" t="inlineStr">
         <is>
           <t>LITTERALIS</t>
         </is>
       </c>
-      <c r="E15" s="14" t="inlineStr">
-        <is>
-          <t>Projet</t>
-        </is>
-      </c>
-      <c r="F15" s="14" t="n">
+      <c r="E19" s="14" t="inlineStr">
+        <is>
+          <t>Projet</t>
+        </is>
+      </c>
+      <c r="F19" s="14" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="27" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="27" t="inlineStr">
         <is>
           <t>PDMDEP-5596</t>
         </is>
       </c>
-      <c r="B16" s="27" t="inlineStr">
+      <c r="B20" s="27" t="inlineStr">
         <is>
           <t>[IVRY-SUR-SEINE - GEODP TLPE/Voirie/Terrasse] GEODP V2</t>
         </is>
       </c>
-      <c r="C16" s="27" t="inlineStr">
+      <c r="C20" s="27" t="inlineStr">
         <is>
           <t>IVRY-SUR-SEINE</t>
         </is>
       </c>
-      <c r="D16" s="27" t="inlineStr">
+      <c r="D20" s="27" t="inlineStr">
         <is>
           <t>GEODP</t>
         </is>
       </c>
-      <c r="E16" s="27" t="inlineStr">
+      <c r="E20" s="27" t="inlineStr">
         <is>
           <t>Rework</t>
         </is>
       </c>
-      <c r="F16" s="27" t="n">
+      <c r="F20" s="27" t="n">
         <v>34</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="27" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="27" t="inlineStr">
         <is>
           <t>PDMDEP-16116</t>
         </is>
       </c>
-      <c r="B17" s="27" t="inlineStr">
+      <c r="B21" s="27" t="inlineStr">
         <is>
           <t>[CD 01] MV + réinstal serveur + flux + publi + TDC SIG et AM</t>
         </is>
       </c>
-      <c r="C17" s="27" t="inlineStr">
+      <c r="C21" s="27" t="inlineStr">
         <is>
           <t>CD 01</t>
         </is>
       </c>
-      <c r="D17" s="27" t="inlineStr">
+      <c r="D21" s="27" t="inlineStr">
         <is>
           <t>LITTERALIS</t>
         </is>
       </c>
-      <c r="E17" s="27" t="inlineStr">
+      <c r="E21" s="27" t="inlineStr">
         <is>
           <t>Rework</t>
         </is>
       </c>
-      <c r="F17" s="27" t="n">
+      <c r="F21" s="27" t="n">
         <v>24</v>
       </c>
     </row>
-    <row r="18"/>
-    <row r="19">
-      <c r="A19" s="17" t="inlineStr">
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" s="17" t="inlineStr">
         <is>
           <t>TOTAL projets clôturés</t>
         </is>
       </c>
-      <c r="B19" s="17" t="n"/>
-      <c r="C19" s="17" t="n"/>
-      <c r="D19" s="17" t="n"/>
-      <c r="E19" s="17" t="n"/>
-      <c r="F19" s="17" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="28" t="inlineStr">
+      <c r="B23" s="17" t="n"/>
+      <c r="C23" s="17" t="n"/>
+      <c r="D23" s="17" t="n"/>
+      <c r="E23" s="17" t="n"/>
+      <c r="F23" s="17" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="28" t="inlineStr">
         <is>
           <t>TOTAL rework clôturés</t>
         </is>
       </c>
-      <c r="B20" s="28" t="n"/>
-      <c r="C20" s="28" t="n"/>
-      <c r="D20" s="28" t="n"/>
-      <c r="E20" s="28" t="n"/>
-      <c r="F20" s="28" t="n">
+      <c r="B24" s="28" t="n"/>
+      <c r="C24" s="28" t="n"/>
+      <c r="D24" s="28" t="n"/>
+      <c r="E24" s="28" t="n"/>
+      <c r="F24" s="28" t="n">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
MAJ pipeline 2026-07-29 14:52
</commit_message>
<xml_diff>
--- a/jira_export_2026-07-29.xlsx
+++ b/jira_export_2026-07-29.xlsx
@@ -732,7 +732,7 @@
     <row r="7" ht="26" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>63,512 €</t>
+          <t>64,023 €</t>
         </is>
       </c>
       <c r="B7" s="7" t="n"/>
@@ -746,7 +746,7 @@
       <c r="F7" s="7" t="n"/>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>66.9%</t>
+          <t>67.4%</t>
         </is>
       </c>
       <c r="H7" s="7" t="n"/>
@@ -772,7 +772,7 @@
     <row r="11" ht="26" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>22,893 €</t>
+          <t>23,404 €</t>
         </is>
       </c>
       <c r="B11" s="7" t="n"/>
@@ -827,7 +827,7 @@
     <row r="16" ht="26" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>568 h</t>
+          <t>570 h</t>
         </is>
       </c>
       <c r="B16" s="7" t="n"/>
@@ -841,7 +841,7 @@
       <c r="F16" s="7" t="n"/>
       <c r="G16" s="9" t="inlineStr">
         <is>
-          <t>71.0%</t>
+          <t>71.3%</t>
         </is>
       </c>
       <c r="H16" s="7" t="n"/>
@@ -912,7 +912,7 @@
       <c r="F25" s="7" t="n"/>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>252</t>
+          <t>255</t>
         </is>
       </c>
       <c r="H25" s="7" t="n"/>
@@ -12375,7 +12375,7 @@
         <v>19</v>
       </c>
       <c r="K164" s="15" t="n">
-        <v>3.62</v>
+        <v>3.75</v>
       </c>
       <c r="L164" s="15" t="inlineStr">
         <is>
@@ -12445,7 +12445,7 @@
         <v>19</v>
       </c>
       <c r="K165" s="12" t="n">
-        <v>3.62</v>
+        <v>3.75</v>
       </c>
       <c r="L165" s="12" t="inlineStr">
         <is>
@@ -12709,7 +12709,7 @@
         <v>27</v>
       </c>
       <c r="K169" s="12" t="n">
-        <v>1.5</v>
+        <v>1.75</v>
       </c>
       <c r="L169" s="12" t="inlineStr">
         <is>
@@ -13639,7 +13639,7 @@
         <v>2</v>
       </c>
       <c r="K184" s="15" t="n">
-        <v>0.5</v>
+        <v>1.75</v>
       </c>
       <c r="L184" s="15" t="inlineStr">
         <is>
@@ -13654,11 +13654,11 @@
       <c r="N184" s="16" t="n">
         <v>510.6</v>
       </c>
-      <c r="O184" s="17" t="n">
-        <v>170.2</v>
+      <c r="O184" s="16" t="n">
+        <v>680.8</v>
       </c>
       <c r="P184" s="16" t="n">
-        <v>340.4</v>
+        <v>389.03</v>
       </c>
     </row>
     <row r="185">
@@ -13951,10 +13951,10 @@
         <v>62442.1</v>
       </c>
       <c r="O190" s="19" t="n">
-        <v>63512.49500000001</v>
+        <v>64023.09500000001</v>
       </c>
       <c r="P190" s="19" t="n">
-        <v>183.56</v>
+        <v>184.1</v>
       </c>
     </row>
   </sheetData>
@@ -15172,7 +15172,7 @@
         </is>
       </c>
       <c r="B5" s="15" t="n">
-        <v>196.25</v>
+        <v>198</v>
       </c>
       <c r="C5" s="15" t="n">
         <v>35</v>
@@ -15181,7 +15181,7 @@
         <v>3.5</v>
       </c>
       <c r="E5" s="15" t="n">
-        <v>234.75</v>
+        <v>236.5</v>
       </c>
       <c r="F5" s="15" t="n">
         <v>68.5</v>
@@ -15191,7 +15191,7 @@
       </c>
       <c r="H5" s="22" t="inlineStr">
         <is>
-          <t>48.3%</t>
+          <t>48.6%</t>
         </is>
       </c>
     </row>
@@ -15233,7 +15233,7 @@
         </is>
       </c>
       <c r="B8" s="24" t="n">
-        <v>129.08</v>
+        <v>129.33</v>
       </c>
     </row>
   </sheetData>
@@ -15318,10 +15318,10 @@
         </is>
       </c>
       <c r="B5" s="25" t="n">
-        <v>387821</v>
+        <v>387310</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>129704</v>
+        <v>129194</v>
       </c>
       <c r="D5" s="25" t="n">
         <v>258116</v>
@@ -15343,10 +15343,10 @@
         </is>
       </c>
       <c r="B6" s="26" t="n">
-        <v>176062</v>
+        <v>175551</v>
       </c>
       <c r="C6" s="26" t="n">
-        <v>70667</v>
+        <v>70156</v>
       </c>
       <c r="D6" s="26" t="n">
         <v>105395</v>
@@ -15397,7 +15397,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -15421,7 +15421,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Épics créées ce mois — 18 commande(s)</t>
+          <t>Épics créées ce mois — 19 commande(s)</t>
         </is>
       </c>
     </row>
@@ -15476,12 +15476,12 @@
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
         <is>
-          <t>PDMDEP-34791</t>
+          <t>PDMDEP-34825</t>
         </is>
       </c>
       <c r="B5" s="15" t="inlineStr">
         <is>
-          <t>PDMDEP-34782</t>
+          <t>PDMDEP-34819</t>
         </is>
       </c>
       <c r="C5" s="15" t="inlineStr">
@@ -15491,7 +15491,7 @@
       </c>
       <c r="D5" s="15" t="inlineStr">
         <is>
-          <t>MAIRIE DE SAINT-ISMIER</t>
+          <t>Ville de Bourges</t>
         </is>
       </c>
       <c r="E5" s="15" t="inlineStr">
@@ -15501,7 +15501,7 @@
       </c>
       <c r="F5" s="15" t="inlineStr">
         <is>
-          <t>Nouveau déploiement</t>
+          <t>Migration</t>
         </is>
       </c>
       <c r="G5" s="15" t="inlineStr">
@@ -15511,11 +15511,11 @@
       </c>
       <c r="H5" s="15" t="inlineStr">
         <is>
-          <t>00177122</t>
+          <t>00177218</t>
         </is>
       </c>
       <c r="I5" s="26" t="n">
-        <v>2146.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -16061,22 +16061,22 @@
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>PDMDEP-34396</t>
+          <t>PDMDEP-34791</t>
         </is>
       </c>
       <c r="B18" s="12" t="inlineStr">
         <is>
-          <t>PDMDEP-34390</t>
+          <t>PDMDEP-34782</t>
         </is>
       </c>
       <c r="C18" s="12" t="inlineStr">
         <is>
-          <t>01/07/2026</t>
+          <t>29/07/2026</t>
         </is>
       </c>
       <c r="D18" s="12" t="inlineStr">
         <is>
-          <t>Commune Le THOR</t>
+          <t>MAIRIE DE SAINT-ISMIER</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
@@ -16086,7 +16086,7 @@
       </c>
       <c r="F18" s="12" t="inlineStr">
         <is>
-          <t>Vente additionnelle</t>
+          <t>Nouveau déploiement</t>
         </is>
       </c>
       <c r="G18" s="12" t="inlineStr">
@@ -16096,37 +16096,37 @@
       </c>
       <c r="H18" s="12" t="inlineStr">
         <is>
-          <t>00171793</t>
+          <t>00177122</t>
         </is>
       </c>
       <c r="I18" s="27" t="n">
-        <v>250</v>
+        <v>2146.5</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>PDMDEP-34722</t>
+          <t>PDMDEP-34396</t>
         </is>
       </c>
       <c r="B19" s="15" t="inlineStr">
         <is>
-          <t>PDMDEP-34718</t>
+          <t>PDMDEP-34390</t>
         </is>
       </c>
       <c r="C19" s="15" t="inlineStr">
         <is>
-          <t>24/07/2026</t>
+          <t>01/07/2026</t>
         </is>
       </c>
       <c r="D19" s="15" t="inlineStr">
         <is>
-          <t>VILLE DE VILLEURBANNE</t>
+          <t>Commune Le THOR</t>
         </is>
       </c>
       <c r="E19" s="15" t="inlineStr">
         <is>
-          <t>LITTERALIS</t>
+          <t>GEODP</t>
         </is>
       </c>
       <c r="F19" s="15" t="inlineStr">
@@ -16141,32 +16141,32 @@
       </c>
       <c r="H19" s="15" t="inlineStr">
         <is>
-          <t>00176875</t>
+          <t>00171793</t>
         </is>
       </c>
       <c r="I19" s="26" t="n">
-        <v>2800</v>
+        <v>250</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t>PDMDEP-34499</t>
+          <t>PDMDEP-34722</t>
         </is>
       </c>
       <c r="B20" s="12" t="inlineStr">
         <is>
-          <t>PDMDEP-34495</t>
+          <t>PDMDEP-34718</t>
         </is>
       </c>
       <c r="C20" s="12" t="inlineStr">
         <is>
-          <t>07/07/2026</t>
+          <t>24/07/2026</t>
         </is>
       </c>
       <c r="D20" s="12" t="inlineStr">
         <is>
-          <t>COMMUNE DE CLICHY</t>
+          <t>VILLE DE VILLEURBANNE</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
@@ -16186,32 +16186,32 @@
       </c>
       <c r="H20" s="12" t="inlineStr">
         <is>
-          <t>00172678</t>
+          <t>00176875</t>
         </is>
       </c>
       <c r="I20" s="27" t="n">
-        <v>4300</v>
+        <v>2800</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>PDMDEP-34778</t>
+          <t>PDMDEP-34499</t>
         </is>
       </c>
       <c r="B21" s="15" t="inlineStr">
         <is>
-          <t>PSC-1315</t>
+          <t>PDMDEP-34495</t>
         </is>
       </c>
       <c r="C21" s="15" t="inlineStr">
         <is>
-          <t>08/07/2026</t>
+          <t>07/07/2026</t>
         </is>
       </c>
       <c r="D21" s="15" t="inlineStr">
         <is>
-          <t>Rang-du-Fliers</t>
+          <t>COMMUNE DE CLICHY</t>
         </is>
       </c>
       <c r="E21" s="15" t="inlineStr">
@@ -16219,83 +16219,107 @@
           <t>LITTERALIS</t>
         </is>
       </c>
-      <c r="F21" s="15" t="inlineStr"/>
-      <c r="G21" s="15" t="inlineStr"/>
-      <c r="H21" s="15" t="inlineStr"/>
+      <c r="F21" s="15" t="inlineStr">
+        <is>
+          <t>Vente additionnelle</t>
+        </is>
+      </c>
+      <c r="G21" s="15" t="inlineStr">
+        <is>
+          <t>Services</t>
+        </is>
+      </c>
+      <c r="H21" s="15" t="inlineStr">
+        <is>
+          <t>00172678</t>
+        </is>
+      </c>
       <c r="I21" s="26" t="n">
-        <v>500</v>
+        <v>4300</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
+          <t>PDMDEP-34778</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>PSC-1315</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>Rang-du-Fliers</t>
+        </is>
+      </c>
+      <c r="E22" s="12" t="inlineStr">
+        <is>
+          <t>LITTERALIS</t>
+        </is>
+      </c>
+      <c r="F22" s="12" t="inlineStr"/>
+      <c r="G22" s="12" t="inlineStr"/>
+      <c r="H22" s="12" t="inlineStr"/>
+      <c r="I22" s="27" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="inlineStr">
+        <is>
           <t>PDMDEP-34654</t>
         </is>
       </c>
-      <c r="B22" s="12" t="inlineStr">
+      <c r="B23" s="15" t="inlineStr">
         <is>
           <t>PDMDEP-34650</t>
         </is>
       </c>
-      <c r="C22" s="12" t="inlineStr">
+      <c r="C23" s="15" t="inlineStr">
         <is>
           <t>21/07/2026</t>
         </is>
       </c>
-      <c r="D22" s="12" t="inlineStr">
+      <c r="D23" s="15" t="inlineStr">
         <is>
           <t>DEPARTEMENT DE L AIN (CD 01)</t>
         </is>
       </c>
-      <c r="E22" s="12" t="inlineStr">
+      <c r="E23" s="15" t="inlineStr">
         <is>
           <t>LITTERALIS</t>
         </is>
       </c>
-      <c r="F22" s="12" t="inlineStr">
+      <c r="F23" s="15" t="inlineStr">
         <is>
           <t>Vente additionnelle</t>
         </is>
       </c>
-      <c r="G22" s="12" t="inlineStr">
+      <c r="G23" s="15" t="inlineStr">
         <is>
           <t>Services</t>
         </is>
       </c>
-      <c r="H22" s="12" t="inlineStr">
+      <c r="H23" s="15" t="inlineStr">
         <is>
           <t>00176582</t>
         </is>
       </c>
-      <c r="I22" s="27" t="n">
+      <c r="I23" s="26" t="n">
         <v>495</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="18" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B23" s="18" t="n"/>
-      <c r="C23" s="18" t="n"/>
-      <c r="D23" s="18" t="n"/>
-      <c r="E23" s="18" t="n"/>
-      <c r="F23" s="18" t="n"/>
-      <c r="G23" s="18" t="n"/>
-      <c r="H23" s="18" t="inlineStr">
-        <is>
-          <t>18 commande(s)</t>
-        </is>
-      </c>
-      <c r="I23" s="25" t="n">
-        <v>38784</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="18" t="inlineStr">
         <is>
-          <t>dont Littéralis</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="B24" s="18" t="n"/>
@@ -16306,17 +16330,17 @@
       <c r="G24" s="18" t="n"/>
       <c r="H24" s="18" t="inlineStr">
         <is>
-          <t>4 commande(s)</t>
+          <t>19 commande(s)</t>
         </is>
       </c>
       <c r="I24" s="25" t="n">
-        <v>8095</v>
+        <v>38784</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="18" t="inlineStr">
         <is>
-          <t>dont GEODP</t>
+          <t>dont Littéralis</t>
         </is>
       </c>
       <c r="B25" s="18" t="n"/>
@@ -16327,10 +16351,31 @@
       <c r="G25" s="18" t="n"/>
       <c r="H25" s="18" t="inlineStr">
         <is>
-          <t>14 commande(s)</t>
+          <t>4 commande(s)</t>
         </is>
       </c>
       <c r="I25" s="25" t="n">
+        <v>8095</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="18" t="inlineStr">
+        <is>
+          <t>dont GEODP</t>
+        </is>
+      </c>
+      <c r="B26" s="18" t="n"/>
+      <c r="C26" s="18" t="n"/>
+      <c r="D26" s="18" t="n"/>
+      <c r="E26" s="18" t="n"/>
+      <c r="F26" s="18" t="n"/>
+      <c r="G26" s="18" t="n"/>
+      <c r="H26" s="18" t="inlineStr">
+        <is>
+          <t>15 commande(s)</t>
+        </is>
+      </c>
+      <c r="I26" s="25" t="n">
         <v>30689</v>
       </c>
     </row>

</xml_diff>

<commit_message>
MAJ pipeline 2026-07-29 18:04
</commit_message>
<xml_diff>
--- a/jira_export_2026-07-29.xlsx
+++ b/jira_export_2026-07-29.xlsx
@@ -827,7 +827,7 @@
     <row r="16" ht="26" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>570 h</t>
+          <t>576 h</t>
         </is>
       </c>
       <c r="B16" s="7" t="n"/>
@@ -841,7 +841,7 @@
       <c r="F16" s="7" t="n"/>
       <c r="G16" s="9" t="inlineStr">
         <is>
-          <t>71.3%</t>
+          <t>72.0%</t>
         </is>
       </c>
       <c r="H16" s="7" t="n"/>
@@ -912,7 +912,7 @@
       <c r="F25" s="7" t="n"/>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>256</t>
         </is>
       </c>
       <c r="H25" s="7" t="n"/>
@@ -2609,7 +2609,7 @@
         <v>1</v>
       </c>
       <c r="K26" s="15" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L26" s="15" t="inlineStr"/>
       <c r="M26" s="15" t="inlineStr"/>
@@ -5177,7 +5177,7 @@
         <v>2</v>
       </c>
       <c r="K62" s="15" t="n">
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="L62" s="15" t="inlineStr">
         <is>
@@ -5249,7 +5249,7 @@
         <v>2</v>
       </c>
       <c r="K63" s="12" t="n">
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="L63" s="12" t="inlineStr">
         <is>
@@ -5268,7 +5268,7 @@
         <v>224</v>
       </c>
       <c r="P63" s="13" t="n">
-        <v>298.67</v>
+        <v>179.2</v>
       </c>
     </row>
     <row r="64">
@@ -11777,7 +11777,7 @@
         <v>16</v>
       </c>
       <c r="K155" s="12" t="n">
-        <v>2.5</v>
+        <v>2.75</v>
       </c>
       <c r="L155" s="12" t="inlineStr"/>
       <c r="M155" s="12" t="inlineStr"/>
@@ -13217,7 +13217,7 @@
         <v>34</v>
       </c>
       <c r="K177" s="12" t="n">
-        <v>1.75</v>
+        <v>2.75</v>
       </c>
       <c r="L177" s="12" t="inlineStr">
         <is>
@@ -13954,7 +13954,7 @@
         <v>64023.09500000001</v>
       </c>
       <c r="P190" s="19" t="n">
-        <v>184.1</v>
+        <v>182.66</v>
       </c>
     </row>
   </sheetData>
@@ -15172,16 +15172,16 @@
         </is>
       </c>
       <c r="B5" s="15" t="n">
-        <v>198</v>
+        <v>199.25</v>
       </c>
       <c r="C5" s="15" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D5" s="15" t="n">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="E5" s="15" t="n">
-        <v>236.5</v>
+        <v>239.25</v>
       </c>
       <c r="F5" s="15" t="n">
         <v>68.5</v>
@@ -15191,7 +15191,7 @@
       </c>
       <c r="H5" s="22" t="inlineStr">
         <is>
-          <t>48.6%</t>
+          <t>49.2%</t>
         </is>
       </c>
     </row>
@@ -15233,7 +15233,7 @@
         </is>
       </c>
       <c r="B8" s="24" t="n">
-        <v>129.33</v>
+        <v>132.58</v>
       </c>
     </row>
   </sheetData>
@@ -15397,7 +15397,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -15421,7 +15421,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Épics créées ce mois — 19 commande(s)</t>
+          <t>Épics créées ce mois — 20 commande(s)</t>
         </is>
       </c>
     </row>
@@ -15476,22 +15476,22 @@
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
         <is>
-          <t>PDMDEP-34825</t>
+          <t>PDMDEP-34396</t>
         </is>
       </c>
       <c r="B5" s="15" t="inlineStr">
         <is>
-          <t>PDMDEP-34819</t>
+          <t>PDMDEP-34390</t>
         </is>
       </c>
       <c r="C5" s="15" t="inlineStr">
         <is>
-          <t>29/07/2026</t>
+          <t>01/07/2026</t>
         </is>
       </c>
       <c r="D5" s="15" t="inlineStr">
         <is>
-          <t>Ville de Bourges</t>
+          <t>Commune Le THOR</t>
         </is>
       </c>
       <c r="E5" s="15" t="inlineStr">
@@ -15501,7 +15501,7 @@
       </c>
       <c r="F5" s="15" t="inlineStr">
         <is>
-          <t>Migration</t>
+          <t>Vente additionnelle</t>
         </is>
       </c>
       <c r="G5" s="15" t="inlineStr">
@@ -15511,32 +15511,32 @@
       </c>
       <c r="H5" s="15" t="inlineStr">
         <is>
-          <t>00177218</t>
+          <t>00171793</t>
         </is>
       </c>
       <c r="I5" s="26" t="n">
-        <v>0</v>
+        <v>250</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
         <is>
-          <t>PDMDEP-34466</t>
+          <t>PDMDEP-34825</t>
         </is>
       </c>
       <c r="B6" s="12" t="inlineStr">
         <is>
-          <t>PDMDEP-34457</t>
+          <t>PDMDEP-34819</t>
         </is>
       </c>
       <c r="C6" s="12" t="inlineStr">
         <is>
-          <t>06/07/2026</t>
+          <t>29/07/2026</t>
         </is>
       </c>
       <c r="D6" s="12" t="inlineStr">
         <is>
-          <t>Commune de La Flèche</t>
+          <t>Ville de Bourges</t>
         </is>
       </c>
       <c r="E6" s="12" t="inlineStr">
@@ -15556,32 +15556,32 @@
       </c>
       <c r="H6" s="12" t="inlineStr">
         <is>
-          <t>00172594</t>
+          <t>00177218</t>
         </is>
       </c>
       <c r="I6" s="27" t="n">
-        <v>4475</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
         <is>
-          <t>PDMDEP-34481</t>
+          <t>PDMDEP-34791</t>
         </is>
       </c>
       <c r="B7" s="15" t="inlineStr">
         <is>
-          <t>PDMDEP-34475</t>
+          <t>PDMDEP-34782</t>
         </is>
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>06/07/2026</t>
+          <t>29/07/2026</t>
         </is>
       </c>
       <c r="D7" s="15" t="inlineStr">
         <is>
-          <t>Mairie de Pontcharra</t>
+          <t>MAIRIE DE SAINT-ISMIER</t>
         </is>
       </c>
       <c r="E7" s="15" t="inlineStr">
@@ -15591,7 +15591,7 @@
       </c>
       <c r="F7" s="15" t="inlineStr">
         <is>
-          <t>Migration</t>
+          <t>Nouveau déploiement</t>
         </is>
       </c>
       <c r="G7" s="15" t="inlineStr">
@@ -15601,32 +15601,32 @@
       </c>
       <c r="H7" s="15" t="inlineStr">
         <is>
-          <t>00172611</t>
+          <t>00177122</t>
         </is>
       </c>
       <c r="I7" s="26" t="n">
-        <v>1050</v>
+        <v>2146.5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>PDMDEP-34527</t>
+          <t>PDMDEP-34466</t>
         </is>
       </c>
       <c r="B8" s="12" t="inlineStr">
         <is>
-          <t>PDMDEP-34521</t>
+          <t>PDMDEP-34457</t>
         </is>
       </c>
       <c r="C8" s="12" t="inlineStr">
         <is>
-          <t>09/07/2026</t>
+          <t>06/07/2026</t>
         </is>
       </c>
       <c r="D8" s="12" t="inlineStr">
         <is>
-          <t>COMMUNE DE FRONTON</t>
+          <t>Commune de La Flèche</t>
         </is>
       </c>
       <c r="E8" s="12" t="inlineStr">
@@ -15636,7 +15636,7 @@
       </c>
       <c r="F8" s="12" t="inlineStr">
         <is>
-          <t>Vente additionnelle</t>
+          <t>Migration</t>
         </is>
       </c>
       <c r="G8" s="12" t="inlineStr">
@@ -15646,32 +15646,32 @@
       </c>
       <c r="H8" s="12" t="inlineStr">
         <is>
-          <t>00173007</t>
+          <t>00172594</t>
         </is>
       </c>
       <c r="I8" s="27" t="n">
-        <v>500</v>
+        <v>4475</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="15" t="inlineStr">
         <is>
-          <t>PDMDEP-34545</t>
+          <t>PDMDEP-34768</t>
         </is>
       </c>
       <c r="B9" s="15" t="inlineStr">
         <is>
-          <t>PDMDEP-34537</t>
+          <t>PDMDEP-34761</t>
         </is>
       </c>
       <c r="C9" s="15" t="inlineStr">
         <is>
-          <t>13/07/2026</t>
+          <t>28/07/2026</t>
         </is>
       </c>
       <c r="D9" s="15" t="inlineStr">
         <is>
-          <t>COMMUNE DE BRON</t>
+          <t>COMMUNE DU PUY EN VELAY</t>
         </is>
       </c>
       <c r="E9" s="15" t="inlineStr">
@@ -15681,7 +15681,7 @@
       </c>
       <c r="F9" s="15" t="inlineStr">
         <is>
-          <t>Vente additionnelle</t>
+          <t>Migration</t>
         </is>
       </c>
       <c r="G9" s="15" t="inlineStr">
@@ -15691,32 +15691,32 @@
       </c>
       <c r="H9" s="15" t="inlineStr">
         <is>
-          <t>00173172</t>
+          <t>00177029</t>
         </is>
       </c>
       <c r="I9" s="26" t="n">
-        <v>1000</v>
+        <v>5585</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="12" t="inlineStr">
         <is>
-          <t>PDMDEP-34589</t>
+          <t>PDMDEP-34481</t>
         </is>
       </c>
       <c r="B10" s="12" t="inlineStr">
         <is>
-          <t>PDMDEP-34580</t>
+          <t>PDMDEP-34475</t>
         </is>
       </c>
       <c r="C10" s="12" t="inlineStr">
         <is>
-          <t>16/07/2026</t>
+          <t>06/07/2026</t>
         </is>
       </c>
       <c r="D10" s="12" t="inlineStr">
         <is>
-          <t>COMMUNE DE RIEZ</t>
+          <t>Mairie de Pontcharra</t>
         </is>
       </c>
       <c r="E10" s="12" t="inlineStr">
@@ -15736,32 +15736,32 @@
       </c>
       <c r="H10" s="12" t="inlineStr">
         <is>
-          <t>00176128</t>
+          <t>00172611</t>
         </is>
       </c>
       <c r="I10" s="27" t="n">
-        <v>1300</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="15" t="inlineStr">
         <is>
-          <t>PDMDEP-34621</t>
+          <t>PDMDEP-34701</t>
         </is>
       </c>
       <c r="B11" s="15" t="inlineStr">
         <is>
-          <t>PDMDEP-34613</t>
+          <t>PDMDEP-34694</t>
         </is>
       </c>
       <c r="C11" s="15" t="inlineStr">
         <is>
-          <t>20/07/2026</t>
+          <t>22/07/2026</t>
         </is>
       </c>
       <c r="D11" s="15" t="inlineStr">
         <is>
-          <t>COMMUNE DE FORT-DE-FRANCE</t>
+          <t>Commune du Tampon</t>
         </is>
       </c>
       <c r="E11" s="15" t="inlineStr">
@@ -15771,7 +15771,7 @@
       </c>
       <c r="F11" s="15" t="inlineStr">
         <is>
-          <t>Vente additionnelle</t>
+          <t>Migration</t>
         </is>
       </c>
       <c r="G11" s="15" t="inlineStr">
@@ -15781,32 +15781,32 @@
       </c>
       <c r="H11" s="15" t="inlineStr">
         <is>
-          <t>00176431</t>
+          <t>00176675</t>
         </is>
       </c>
       <c r="I11" s="26" t="n">
-        <v>2000</v>
+        <v>3947.5</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
         <is>
-          <t>PDMDEP-34420</t>
+          <t>PDMDEP-34683</t>
         </is>
       </c>
       <c r="B12" s="12" t="inlineStr">
         <is>
-          <t>PDMDEP-34411</t>
+          <t>PDMDEP-34676</t>
         </is>
       </c>
       <c r="C12" s="12" t="inlineStr">
         <is>
-          <t>02/07/2026</t>
+          <t>22/07/2026</t>
         </is>
       </c>
       <c r="D12" s="12" t="inlineStr">
         <is>
-          <t>MAIRIE DE MAIZIERES LES METZ</t>
+          <t>Commune des Ponts de Ce</t>
         </is>
       </c>
       <c r="E12" s="12" t="inlineStr">
@@ -15826,32 +15826,32 @@
       </c>
       <c r="H12" s="12" t="inlineStr">
         <is>
-          <t>00172317</t>
+          <t>00176614</t>
         </is>
       </c>
       <c r="I12" s="27" t="n">
-        <v>2035</v>
+        <v>2150</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>PDMDEP-34640</t>
+          <t>PDMDEP-34666</t>
         </is>
       </c>
       <c r="B13" s="15" t="inlineStr">
         <is>
-          <t>PDMDEP-34631</t>
+          <t>PDMDEP-34659</t>
         </is>
       </c>
       <c r="C13" s="15" t="inlineStr">
         <is>
-          <t>21/07/2026</t>
+          <t>22/07/2026</t>
         </is>
       </c>
       <c r="D13" s="15" t="inlineStr">
         <is>
-          <t>COMMUNE DE SAINT-HILAIRE-DE-RIEZ</t>
+          <t>Commune des Ponts de Ce</t>
         </is>
       </c>
       <c r="E13" s="15" t="inlineStr">
@@ -15861,7 +15861,7 @@
       </c>
       <c r="F13" s="15" t="inlineStr">
         <is>
-          <t>Nouveau déploiement</t>
+          <t>Migration</t>
         </is>
       </c>
       <c r="G13" s="15" t="inlineStr">
@@ -15871,32 +15871,32 @@
       </c>
       <c r="H13" s="15" t="inlineStr">
         <is>
-          <t>00176477</t>
+          <t>00176614</t>
         </is>
       </c>
       <c r="I13" s="26" t="n">
-        <v>2250</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
         <is>
-          <t>PDMDEP-34666</t>
+          <t>PDMDEP-34420</t>
         </is>
       </c>
       <c r="B14" s="12" t="inlineStr">
         <is>
-          <t>PDMDEP-34659</t>
+          <t>PDMDEP-34411</t>
         </is>
       </c>
       <c r="C14" s="12" t="inlineStr">
         <is>
-          <t>22/07/2026</t>
+          <t>02/07/2026</t>
         </is>
       </c>
       <c r="D14" s="12" t="inlineStr">
         <is>
-          <t>Commune des Ponts de Ce</t>
+          <t>MAIRIE DE MAIZIERES LES METZ</t>
         </is>
       </c>
       <c r="E14" s="12" t="inlineStr">
@@ -15916,32 +15916,32 @@
       </c>
       <c r="H14" s="12" t="inlineStr">
         <is>
-          <t>00176614</t>
+          <t>00172317</t>
         </is>
       </c>
       <c r="I14" s="27" t="n">
-        <v>2000</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>PDMDEP-34683</t>
+          <t>PDMDEP-34640</t>
         </is>
       </c>
       <c r="B15" s="15" t="inlineStr">
         <is>
-          <t>PDMDEP-34676</t>
+          <t>PDMDEP-34631</t>
         </is>
       </c>
       <c r="C15" s="15" t="inlineStr">
         <is>
-          <t>22/07/2026</t>
+          <t>21/07/2026</t>
         </is>
       </c>
       <c r="D15" s="15" t="inlineStr">
         <is>
-          <t>Commune des Ponts de Ce</t>
+          <t>COMMUNE DE SAINT-HILAIRE-DE-RIEZ</t>
         </is>
       </c>
       <c r="E15" s="15" t="inlineStr">
@@ -15951,7 +15951,7 @@
       </c>
       <c r="F15" s="15" t="inlineStr">
         <is>
-          <t>Migration</t>
+          <t>Nouveau déploiement</t>
         </is>
       </c>
       <c r="G15" s="15" t="inlineStr">
@@ -15961,32 +15961,32 @@
       </c>
       <c r="H15" s="15" t="inlineStr">
         <is>
-          <t>00176614</t>
+          <t>00176477</t>
         </is>
       </c>
       <c r="I15" s="26" t="n">
-        <v>2150</v>
+        <v>2250</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t>PDMDEP-34701</t>
+          <t>PDMDEP-34621</t>
         </is>
       </c>
       <c r="B16" s="12" t="inlineStr">
         <is>
-          <t>PDMDEP-34694</t>
+          <t>PDMDEP-34613</t>
         </is>
       </c>
       <c r="C16" s="12" t="inlineStr">
         <is>
-          <t>22/07/2026</t>
+          <t>20/07/2026</t>
         </is>
       </c>
       <c r="D16" s="12" t="inlineStr">
         <is>
-          <t>Commune du Tampon</t>
+          <t>COMMUNE DE FORT-DE-FRANCE</t>
         </is>
       </c>
       <c r="E16" s="12" t="inlineStr">
@@ -15996,7 +15996,7 @@
       </c>
       <c r="F16" s="12" t="inlineStr">
         <is>
-          <t>Migration</t>
+          <t>Vente additionnelle</t>
         </is>
       </c>
       <c r="G16" s="12" t="inlineStr">
@@ -16006,32 +16006,32 @@
       </c>
       <c r="H16" s="12" t="inlineStr">
         <is>
-          <t>00176675</t>
+          <t>00176431</t>
         </is>
       </c>
       <c r="I16" s="27" t="n">
-        <v>3947.5</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>PDMDEP-34768</t>
+          <t>PDMDEP-34589</t>
         </is>
       </c>
       <c r="B17" s="15" t="inlineStr">
         <is>
-          <t>PDMDEP-34761</t>
+          <t>PDMDEP-34580</t>
         </is>
       </c>
       <c r="C17" s="15" t="inlineStr">
         <is>
-          <t>28/07/2026</t>
+          <t>16/07/2026</t>
         </is>
       </c>
       <c r="D17" s="15" t="inlineStr">
         <is>
-          <t>COMMUNE DU PUY EN VELAY</t>
+          <t>COMMUNE DE RIEZ</t>
         </is>
       </c>
       <c r="E17" s="15" t="inlineStr">
@@ -16051,32 +16051,32 @@
       </c>
       <c r="H17" s="15" t="inlineStr">
         <is>
-          <t>00177029</t>
+          <t>00176128</t>
         </is>
       </c>
       <c r="I17" s="26" t="n">
-        <v>5585</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>PDMDEP-34791</t>
+          <t>PDMDEP-34545</t>
         </is>
       </c>
       <c r="B18" s="12" t="inlineStr">
         <is>
-          <t>PDMDEP-34782</t>
+          <t>PDMDEP-34537</t>
         </is>
       </c>
       <c r="C18" s="12" t="inlineStr">
         <is>
-          <t>29/07/2026</t>
+          <t>13/07/2026</t>
         </is>
       </c>
       <c r="D18" s="12" t="inlineStr">
         <is>
-          <t>MAIRIE DE SAINT-ISMIER</t>
+          <t>COMMUNE DE BRON</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
@@ -16086,7 +16086,7 @@
       </c>
       <c r="F18" s="12" t="inlineStr">
         <is>
-          <t>Nouveau déploiement</t>
+          <t>Vente additionnelle</t>
         </is>
       </c>
       <c r="G18" s="12" t="inlineStr">
@@ -16096,32 +16096,32 @@
       </c>
       <c r="H18" s="12" t="inlineStr">
         <is>
-          <t>00177122</t>
+          <t>00173172</t>
         </is>
       </c>
       <c r="I18" s="27" t="n">
-        <v>2146.5</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>PDMDEP-34396</t>
+          <t>PDMDEP-34527</t>
         </is>
       </c>
       <c r="B19" s="15" t="inlineStr">
         <is>
-          <t>PDMDEP-34390</t>
+          <t>PDMDEP-34521</t>
         </is>
       </c>
       <c r="C19" s="15" t="inlineStr">
         <is>
-          <t>01/07/2026</t>
+          <t>09/07/2026</t>
         </is>
       </c>
       <c r="D19" s="15" t="inlineStr">
         <is>
-          <t>Commune Le THOR</t>
+          <t>COMMUNE DE FRONTON</t>
         </is>
       </c>
       <c r="E19" s="15" t="inlineStr">
@@ -16141,32 +16141,32 @@
       </c>
       <c r="H19" s="15" t="inlineStr">
         <is>
-          <t>00171793</t>
+          <t>00173007</t>
         </is>
       </c>
       <c r="I19" s="26" t="n">
-        <v>250</v>
+        <v>500</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t>PDMDEP-34722</t>
+          <t>PDMDEP-34852</t>
         </is>
       </c>
       <c r="B20" s="12" t="inlineStr">
         <is>
-          <t>PDMDEP-34718</t>
+          <t>PDMDEP-34848</t>
         </is>
       </c>
       <c r="C20" s="12" t="inlineStr">
         <is>
-          <t>24/07/2026</t>
+          <t>29/07/2026</t>
         </is>
       </c>
       <c r="D20" s="12" t="inlineStr">
         <is>
-          <t>VILLE DE VILLEURBANNE</t>
+          <t>COMMUNE DE BRUAY LA BUISSIERE</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
@@ -16186,32 +16186,32 @@
       </c>
       <c r="H20" s="12" t="inlineStr">
         <is>
-          <t>00176875</t>
+          <t>00177232</t>
         </is>
       </c>
       <c r="I20" s="27" t="n">
-        <v>2800</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>PDMDEP-34499</t>
+          <t>PDMDEP-34722</t>
         </is>
       </c>
       <c r="B21" s="15" t="inlineStr">
         <is>
-          <t>PDMDEP-34495</t>
+          <t>PDMDEP-34718</t>
         </is>
       </c>
       <c r="C21" s="15" t="inlineStr">
         <is>
-          <t>07/07/2026</t>
+          <t>24/07/2026</t>
         </is>
       </c>
       <c r="D21" s="15" t="inlineStr">
         <is>
-          <t>COMMUNE DE CLICHY</t>
+          <t>VILLE DE VILLEURBANNE</t>
         </is>
       </c>
       <c r="E21" s="15" t="inlineStr">
@@ -16231,11 +16231,11 @@
       </c>
       <c r="H21" s="15" t="inlineStr">
         <is>
-          <t>00172678</t>
+          <t>00176875</t>
         </is>
       </c>
       <c r="I21" s="26" t="n">
-        <v>4300</v>
+        <v>2800</v>
       </c>
     </row>
     <row r="22">
@@ -16274,73 +16274,97 @@
     <row r="23">
       <c r="A23" s="15" t="inlineStr">
         <is>
+          <t>PDMDEP-34499</t>
+        </is>
+      </c>
+      <c r="B23" s="15" t="inlineStr">
+        <is>
+          <t>PDMDEP-34495</t>
+        </is>
+      </c>
+      <c r="C23" s="15" t="inlineStr">
+        <is>
+          <t>07/07/2026</t>
+        </is>
+      </c>
+      <c r="D23" s="15" t="inlineStr">
+        <is>
+          <t>COMMUNE DE CLICHY</t>
+        </is>
+      </c>
+      <c r="E23" s="15" t="inlineStr">
+        <is>
+          <t>LITTERALIS</t>
+        </is>
+      </c>
+      <c r="F23" s="15" t="inlineStr">
+        <is>
+          <t>Vente additionnelle</t>
+        </is>
+      </c>
+      <c r="G23" s="15" t="inlineStr">
+        <is>
+          <t>Services</t>
+        </is>
+      </c>
+      <c r="H23" s="15" t="inlineStr">
+        <is>
+          <t>00172678</t>
+        </is>
+      </c>
+      <c r="I23" s="26" t="n">
+        <v>4300</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
           <t>PDMDEP-34654</t>
         </is>
       </c>
-      <c r="B23" s="15" t="inlineStr">
+      <c r="B24" s="12" t="inlineStr">
         <is>
           <t>PDMDEP-34650</t>
         </is>
       </c>
-      <c r="C23" s="15" t="inlineStr">
+      <c r="C24" s="12" t="inlineStr">
         <is>
           <t>21/07/2026</t>
         </is>
       </c>
-      <c r="D23" s="15" t="inlineStr">
+      <c r="D24" s="12" t="inlineStr">
         <is>
           <t>DEPARTEMENT DE L AIN (CD 01)</t>
         </is>
       </c>
-      <c r="E23" s="15" t="inlineStr">
+      <c r="E24" s="12" t="inlineStr">
         <is>
           <t>LITTERALIS</t>
         </is>
       </c>
-      <c r="F23" s="15" t="inlineStr">
+      <c r="F24" s="12" t="inlineStr">
         <is>
           <t>Vente additionnelle</t>
         </is>
       </c>
-      <c r="G23" s="15" t="inlineStr">
+      <c r="G24" s="12" t="inlineStr">
         <is>
           <t>Services</t>
         </is>
       </c>
-      <c r="H23" s="15" t="inlineStr">
+      <c r="H24" s="12" t="inlineStr">
         <is>
           <t>00176582</t>
         </is>
       </c>
-      <c r="I23" s="26" t="n">
+      <c r="I24" s="27" t="n">
         <v>495</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="18" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B24" s="18" t="n"/>
-      <c r="C24" s="18" t="n"/>
-      <c r="D24" s="18" t="n"/>
-      <c r="E24" s="18" t="n"/>
-      <c r="F24" s="18" t="n"/>
-      <c r="G24" s="18" t="n"/>
-      <c r="H24" s="18" t="inlineStr">
-        <is>
-          <t>19 commande(s)</t>
-        </is>
-      </c>
-      <c r="I24" s="25" t="n">
-        <v>38784</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="18" t="inlineStr">
         <is>
-          <t>dont Littéralis</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="B25" s="18" t="n"/>
@@ -16351,17 +16375,17 @@
       <c r="G25" s="18" t="n"/>
       <c r="H25" s="18" t="inlineStr">
         <is>
-          <t>4 commande(s)</t>
+          <t>20 commande(s)</t>
         </is>
       </c>
       <c r="I25" s="25" t="n">
-        <v>8095</v>
+        <v>38784</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="18" t="inlineStr">
         <is>
-          <t>dont GEODP</t>
+          <t>dont Littéralis</t>
         </is>
       </c>
       <c r="B26" s="18" t="n"/>
@@ -16372,10 +16396,31 @@
       <c r="G26" s="18" t="n"/>
       <c r="H26" s="18" t="inlineStr">
         <is>
+          <t>5 commande(s)</t>
+        </is>
+      </c>
+      <c r="I26" s="25" t="n">
+        <v>8095</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="18" t="inlineStr">
+        <is>
+          <t>dont GEODP</t>
+        </is>
+      </c>
+      <c r="B27" s="18" t="n"/>
+      <c r="C27" s="18" t="n"/>
+      <c r="D27" s="18" t="n"/>
+      <c r="E27" s="18" t="n"/>
+      <c r="F27" s="18" t="n"/>
+      <c r="G27" s="18" t="n"/>
+      <c r="H27" s="18" t="inlineStr">
+        <is>
           <t>15 commande(s)</t>
         </is>
       </c>
-      <c r="I26" s="25" t="n">
+      <c r="I27" s="25" t="n">
         <v>30689</v>
       </c>
     </row>

</xml_diff>